<commit_message>
Add thesis figures and sweeps, archive unused scripts
- New thesis analyses: stochastic_sweep.py (belief sweep),
  lebanon_summerday.py (four-scenario summer day) and timeseries.py
- Model and sweep updates: deviation-form demand response, 0.01 $/kWh
  price menu, diesel cost 0.224 $/kWh; regenerated outputs
- thesis/: figures as used in the thesis (no titles or in-plot notes,
  larger fonts, shortened labels, two-decimal price axes)
- Archive scenario_analysis.py, loadshift_sweep.py and graphs.py; drop
  the scenario-mismatch stage and --skip-mismatch from run.py
- .gitignore as a whitelist: active .py files, data/*.yaml, output/ and
  thesis/ only; archive/ and loose documents are no longer tracked

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/output/scenario_analysis.xlsx
+++ b/output/scenario_analysis.xlsx
@@ -8,10 +8,10 @@
   </bookViews>
   <sheets>
     <sheet name="summary" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="winter_profit" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="winter_regret" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="winter_sales" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet name="winter_prices" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet name="summer_profit" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="summer_regret" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="summer_sales" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="summer_prices" sheetId="5" state="visible" r:id="rId5"/>
     <sheet name="detail" sheetId="6" state="visible" r:id="rId6"/>
   </sheets>
   <definedNames/>
@@ -435,7 +435,7 @@
     <col width="14" customWidth="1" min="8" max="8"/>
     <col width="18" customWidth="1" min="9" max="9"/>
     <col width="28" customWidth="1" min="10" max="10"/>
-    <col width="22" customWidth="1" min="11" max="11"/>
+    <col width="28" customWidth="1" min="11" max="11"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -491,14 +491,14 @@
       </c>
       <c r="K1" s="1" t="inlineStr">
         <is>
-          <t>cost vs hedged [$]</t>
+          <t>cost vs stochastic commitment [$]</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>winter</t>
+          <t>summer</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
@@ -515,13 +515,13 @@
         <v>0.4</v>
       </c>
       <c r="E2" t="n">
-        <v>55.27734858696385</v>
+        <v>1675.735510873965</v>
       </c>
       <c r="F2" t="n">
-        <v>64.95514390575454</v>
+        <v>1649.87568633307</v>
       </c>
       <c r="G2" t="n">
-        <v>0</v>
+        <v>180.6652719552377</v>
       </c>
       <c r="H2" t="inlineStr">
         <is>
@@ -529,19 +529,19 @@
         </is>
       </c>
       <c r="I2" t="n">
-        <v>4.645221342026389</v>
+        <v>15.39817218019797</v>
       </c>
       <c r="J2" t="n">
-        <v>0.9200112930098641</v>
+        <v>0.7918713614728858</v>
       </c>
       <c r="K2" t="n">
-        <v>0.3628094547848519</v>
+        <v>0</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>winter</t>
+          <t>summer</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
@@ -558,13 +558,13 @@
         <v>0.15</v>
       </c>
       <c r="E3" t="n">
-        <v>96.49851508457135</v>
+        <v>1901.778619953512</v>
       </c>
       <c r="F3" t="n">
-        <v>64.13022890910526</v>
+        <v>1649.87568633307</v>
       </c>
       <c r="G3" t="n">
-        <v>0</v>
+        <v>180.6652719552377</v>
       </c>
       <c r="H3" t="inlineStr">
         <is>
@@ -572,19 +572,19 @@
         </is>
       </c>
       <c r="I3" t="n">
-        <v>3.705432386063777</v>
+        <v>15.39817218019797</v>
       </c>
       <c r="J3" t="n">
-        <v>1.744926289659148</v>
+        <v>0.7918713614728858</v>
       </c>
       <c r="K3" t="n">
-        <v>1.187724451434136</v>
+        <v>0</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>winter</t>
+          <t>summer</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
@@ -601,13 +601,13 @@
         <v>0.2</v>
       </c>
       <c r="E4" t="n">
-        <v>58.74781335549773</v>
+        <v>1672.370747162951</v>
       </c>
       <c r="F4" t="n">
-        <v>65.25201120872106</v>
+        <v>1649.87568633307</v>
       </c>
       <c r="G4" t="n">
-        <v>0</v>
+        <v>180.6652719552377</v>
       </c>
       <c r="H4" t="inlineStr">
         <is>
@@ -615,19 +615,19 @@
         </is>
       </c>
       <c r="I4" t="n">
-        <v>2.919995946517986</v>
+        <v>15.39817218019797</v>
       </c>
       <c r="J4" t="n">
-        <v>0.6231439900433458</v>
+        <v>0.7918713614728858</v>
       </c>
       <c r="K4" t="n">
-        <v>0.06594215181833363</v>
+        <v>0</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>winter</t>
+          <t>summer</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
@@ -644,13 +644,13 @@
         <v>0.1</v>
       </c>
       <c r="E5" t="n">
-        <v>32.08166568020633</v>
+        <v>1351.150369777617</v>
       </c>
       <c r="F5" t="n">
-        <v>63.66863384637695</v>
+        <v>1649.147061207165</v>
       </c>
       <c r="G5" t="n">
-        <v>0</v>
+        <v>183.9658054405357</v>
       </c>
       <c r="H5" t="inlineStr">
         <is>
@@ -658,19 +658,19 @@
         </is>
       </c>
       <c r="I5" t="n">
-        <v>9.289943823697513</v>
+        <v>12.09763869490001</v>
       </c>
       <c r="J5" t="n">
-        <v>2.206521352387455</v>
+        <v>1.520496487377841</v>
       </c>
       <c r="K5" t="n">
-        <v>1.649319514162443</v>
+        <v>0.728625125904955</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>winter</t>
+          <t>summer</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
@@ -687,33 +687,33 @@
         <v>0.05</v>
       </c>
       <c r="E6" t="n">
-        <v>0</v>
+        <v>196.0634441354355</v>
       </c>
       <c r="F6" t="n">
-        <v>-117.441350607779</v>
+        <v>1569.340667200824</v>
       </c>
       <c r="G6" t="n">
-        <v>-221.8718013412653</v>
+        <v>196.0634441354357</v>
       </c>
       <c r="H6" t="inlineStr">
         <is>
-          <t>none</t>
+          <t>full_supply</t>
         </is>
       </c>
       <c r="I6" t="n">
-        <v>365.1888939630039</v>
+        <v>113.6776888270774</v>
       </c>
       <c r="J6" t="n">
-        <v>183.3165058065434</v>
+        <v>81.32689049371879</v>
       </c>
       <c r="K6" t="n">
-        <v>182.7593039683184</v>
+        <v>80.53501913224591</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>winter</t>
+          <t>summer</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
@@ -730,13 +730,13 @@
         <v>0.1</v>
       </c>
       <c r="E7" t="n">
-        <v>143.3170926217407</v>
+        <v>2157.142017348047</v>
       </c>
       <c r="F7" t="n">
-        <v>64.13022890910526</v>
+        <v>1649.87568633307</v>
       </c>
       <c r="G7" t="n">
-        <v>0</v>
+        <v>180.6652719552377</v>
       </c>
       <c r="H7" t="inlineStr">
         <is>
@@ -744,19 +744,19 @@
         </is>
       </c>
       <c r="I7" t="n">
-        <v>3.705432386063777</v>
+        <v>15.39817218019797</v>
       </c>
       <c r="J7" t="n">
-        <v>1.744926289659148</v>
+        <v>0.7918713614728858</v>
       </c>
       <c r="K7" t="n">
-        <v>1.187724451434136</v>
+        <v>0</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>winter</t>
+          <t>summer</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
@@ -766,17 +766,17 @@
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>Hedged (stochastic)</t>
+          <t>Stochastic commitment</t>
         </is>
       </c>
       <c r="E8" t="n">
-        <v>67.3344497940341</v>
+        <v>1649.875686333618</v>
       </c>
       <c r="F8" t="n">
-        <v>65.31795336053939</v>
+        <v>1649.87568633307</v>
       </c>
       <c r="G8" t="n">
-        <v>0</v>
+        <v>180.6652719552377</v>
       </c>
       <c r="H8" t="inlineStr">
         <is>
@@ -784,10 +784,10 @@
         </is>
       </c>
       <c r="I8" t="n">
-        <v>1.592861114561344</v>
+        <v>15.39817218019797</v>
       </c>
       <c r="J8" t="n">
-        <v>0.5572018382250121</v>
+        <v>0.7918713614728858</v>
       </c>
       <c r="K8" t="n">
         <v>0</v>
@@ -796,7 +796,7 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>winter</t>
+          <t>summer</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
@@ -810,7 +810,7 @@
         </is>
       </c>
       <c r="F9" t="n">
-        <v>65.8751551987644</v>
+        <v>1650.667557694543</v>
       </c>
       <c r="J9" t="n">
         <v>0</v>
@@ -819,7 +819,7 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>winter</t>
+          <t>summer</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
@@ -829,11 +829,11 @@
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>perfect foresight - hedged</t>
+          <t>perfect foresight - stochastic commitment</t>
         </is>
       </c>
       <c r="F10" t="n">
-        <v>0.5572018382250121</v>
+        <v>0.7918713614728858</v>
       </c>
     </row>
   </sheetData>
@@ -903,22 +903,22 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>55.27734858696292</v>
+        <v>1675.735510873967</v>
       </c>
       <c r="C2" t="n">
-        <v>93.69818635242842</v>
+        <v>1901.778619953518</v>
       </c>
       <c r="D2" t="n">
-        <v>58.70488182248729</v>
+        <v>1672.370747162953</v>
       </c>
       <c r="E2" t="n">
-        <v>31.81313025636415</v>
+        <v>1350.930742252985</v>
       </c>
       <c r="F2" t="n">
-        <v>0</v>
+        <v>180.6652719552377</v>
       </c>
       <c r="G2" t="n">
-        <v>138.6718712797123</v>
+        <v>2157.142017348049</v>
       </c>
     </row>
     <row r="3">
@@ -928,22 +928,22 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>52.89703753948382</v>
+        <v>1675.735510873967</v>
       </c>
       <c r="C3" t="n">
-        <v>96.49851508456965</v>
+        <v>1901.778619953518</v>
       </c>
       <c r="D3" t="n">
-        <v>56.63652019519108</v>
+        <v>1672.370747162953</v>
       </c>
       <c r="E3" t="n">
-        <v>28.3762332941421</v>
+        <v>1350.930742252985</v>
       </c>
       <c r="F3" t="n">
-        <v>0</v>
+        <v>180.6652719552377</v>
       </c>
       <c r="G3" t="n">
-        <v>143.3170926217387</v>
+        <v>2157.142017348049</v>
       </c>
     </row>
     <row r="4">
@@ -953,22 +953,22 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>55.24405214982986</v>
+        <v>1675.735510873967</v>
       </c>
       <c r="C4" t="n">
-        <v>94.80624361354364</v>
+        <v>1901.778619953518</v>
       </c>
       <c r="D4" t="n">
-        <v>58.74781335549667</v>
+        <v>1672.370747162953</v>
       </c>
       <c r="E4" t="n">
-        <v>31.44181468136175</v>
+        <v>1350.930742252985</v>
       </c>
       <c r="F4" t="n">
-        <v>0</v>
+        <v>180.6652719552377</v>
       </c>
       <c r="G4" t="n">
-        <v>140.3970966752207</v>
+        <v>2157.142017348049</v>
       </c>
     </row>
     <row r="5">
@@ -978,22 +978,22 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>54.67979280268491</v>
+        <v>1675.116383159482</v>
       </c>
       <c r="C5" t="n">
-        <v>90.66008455816774</v>
+        <v>1899.907303522919</v>
       </c>
       <c r="D5" t="n">
-        <v>57.93411296876559</v>
+        <v>1671.495711893862</v>
       </c>
       <c r="E5" t="n">
-        <v>32.08166568020587</v>
+        <v>1351.150369777616</v>
       </c>
       <c r="F5" t="n">
-        <v>0</v>
+        <v>183.9658054405357</v>
       </c>
       <c r="G5" t="n">
-        <v>134.0271487980411</v>
+        <v>2155.019427863739</v>
       </c>
     </row>
     <row r="6">
@@ -1003,22 +1003,22 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>-107.5021054623863</v>
+        <v>1594.80446851474</v>
       </c>
       <c r="C6" t="n">
-        <v>-151.43884576145</v>
+        <v>1801.558144695776</v>
       </c>
       <c r="D6" t="n">
-        <v>-112.0982459944941</v>
+        <v>1589.759955512711</v>
       </c>
       <c r="E6" t="n">
-        <v>-71.17852225581669</v>
+        <v>1290.835619291507</v>
       </c>
       <c r="F6" t="n">
-        <v>0</v>
+        <v>196.0634441354357</v>
       </c>
       <c r="G6" t="n">
-        <v>-221.8718013412653</v>
+        <v>2043.464328520971</v>
       </c>
     </row>
     <row r="7">
@@ -1028,47 +1028,47 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>52.89703753948382</v>
+        <v>1675.735510873967</v>
       </c>
       <c r="C7" t="n">
-        <v>96.49851508456965</v>
+        <v>1901.778619953518</v>
       </c>
       <c r="D7" t="n">
-        <v>56.63652019519108</v>
+        <v>1672.370747162953</v>
       </c>
       <c r="E7" t="n">
-        <v>28.3762332941421</v>
+        <v>1350.930742252985</v>
       </c>
       <c r="F7" t="n">
-        <v>0</v>
+        <v>180.6652719552377</v>
       </c>
       <c r="G7" t="n">
-        <v>143.3170926217387</v>
+        <v>2157.142017348049</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>Hedged (stochastic)</t>
+          <t>Stochastic commitment</t>
         </is>
       </c>
       <c r="B8" t="n">
-        <v>54.98937282651542</v>
+        <v>1675.735510873967</v>
       </c>
       <c r="C8" t="n">
-        <v>95.64030511731534</v>
+        <v>1901.778619953518</v>
       </c>
       <c r="D8" t="n">
-        <v>58.56244295927172</v>
+        <v>1672.370747162953</v>
       </c>
       <c r="E8" t="n">
-        <v>30.91246719763835</v>
+        <v>1350.930742252985</v>
       </c>
       <c r="F8" t="n">
-        <v>0</v>
+        <v>180.6652719552377</v>
       </c>
       <c r="G8" t="n">
-        <v>141.7242315071773</v>
+        <v>2157.142017348049</v>
       </c>
     </row>
     <row r="10">
@@ -1148,19 +1148,19 @@
         <v>0</v>
       </c>
       <c r="C2" t="n">
-        <v>2.800328732141224</v>
+        <v>0</v>
       </c>
       <c r="D2" t="n">
-        <v>0.04293153300938002</v>
+        <v>0</v>
       </c>
       <c r="E2" t="n">
-        <v>0.2685354238417261</v>
+        <v>0.2196275246308232</v>
       </c>
       <c r="F2" t="n">
-        <v>0</v>
+        <v>15.39817218019797</v>
       </c>
       <c r="G2" t="n">
-        <v>4.645221342026389</v>
+        <v>0</v>
       </c>
     </row>
     <row r="3">
@@ -1170,19 +1170,19 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>2.380311047479097</v>
+        <v>0</v>
       </c>
       <c r="C3" t="n">
         <v>0</v>
       </c>
       <c r="D3" t="n">
-        <v>2.111293160305593</v>
+        <v>0</v>
       </c>
       <c r="E3" t="n">
-        <v>3.705432386063777</v>
+        <v>0.2196275246308232</v>
       </c>
       <c r="F3" t="n">
-        <v>0</v>
+        <v>15.39817218019797</v>
       </c>
       <c r="G3" t="n">
         <v>0</v>
@@ -1195,22 +1195,22 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>0.03329643713306041</v>
+        <v>0</v>
       </c>
       <c r="C4" t="n">
-        <v>1.692271471026004</v>
+        <v>0</v>
       </c>
       <c r="D4" t="n">
         <v>0</v>
       </c>
       <c r="E4" t="n">
-        <v>0.6398509988441248</v>
+        <v>0.2196275246308232</v>
       </c>
       <c r="F4" t="n">
-        <v>0</v>
+        <v>15.39817218019797</v>
       </c>
       <c r="G4" t="n">
-        <v>2.919995946517986</v>
+        <v>0</v>
       </c>
     </row>
     <row r="5">
@@ -1220,22 +1220,22 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>0.5975557842780006</v>
+        <v>0.6191277144848755</v>
       </c>
       <c r="C5" t="n">
-        <v>5.838430526401908</v>
+        <v>1.871316430598654</v>
       </c>
       <c r="D5" t="n">
-        <v>0.8137003867310852</v>
+        <v>0.8750352690906311</v>
       </c>
       <c r="E5" t="n">
         <v>0</v>
       </c>
       <c r="F5" t="n">
-        <v>0</v>
+        <v>12.09763869490001</v>
       </c>
       <c r="G5" t="n">
-        <v>9.289943823697513</v>
+        <v>2.122589484309628</v>
       </c>
     </row>
     <row r="6">
@@ -1245,22 +1245,22 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>162.7794540493492</v>
+        <v>80.93104235922647</v>
       </c>
       <c r="C6" t="n">
-        <v>247.9373608460197</v>
+        <v>100.220475257742</v>
       </c>
       <c r="D6" t="n">
-        <v>170.8460593499907</v>
+        <v>82.61079165024194</v>
       </c>
       <c r="E6" t="n">
-        <v>103.2601879360226</v>
+        <v>60.31475048610878</v>
       </c>
       <c r="F6" t="n">
         <v>0</v>
       </c>
       <c r="G6" t="n">
-        <v>365.1888939630039</v>
+        <v>113.6776888270774</v>
       </c>
     </row>
     <row r="7">
@@ -1270,19 +1270,19 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>2.380311047479097</v>
+        <v>0</v>
       </c>
       <c r="C7" t="n">
         <v>0</v>
       </c>
       <c r="D7" t="n">
-        <v>2.111293160305593</v>
+        <v>0</v>
       </c>
       <c r="E7" t="n">
-        <v>3.705432386063777</v>
+        <v>0.2196275246308232</v>
       </c>
       <c r="F7" t="n">
-        <v>0</v>
+        <v>15.39817218019797</v>
       </c>
       <c r="G7" t="n">
         <v>0</v>
@@ -1291,26 +1291,26 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>Hedged (stochastic)</t>
+          <t>Stochastic commitment</t>
         </is>
       </c>
       <c r="B8" t="n">
-        <v>0.2879757604474946</v>
+        <v>0</v>
       </c>
       <c r="C8" t="n">
-        <v>0.8582099672543109</v>
+        <v>0</v>
       </c>
       <c r="D8" t="n">
-        <v>0.185370396224954</v>
+        <v>0</v>
       </c>
       <c r="E8" t="n">
-        <v>1.169198482567523</v>
+        <v>0.2196275246308232</v>
       </c>
       <c r="F8" t="n">
-        <v>0</v>
+        <v>15.39817218019797</v>
       </c>
       <c r="G8" t="n">
-        <v>1.592861114561344</v>
+        <v>0</v>
       </c>
     </row>
     <row r="10">
@@ -1387,22 +1387,22 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>402.0170806324575</v>
+        <v>3307.685534485186</v>
       </c>
       <c r="C2" t="n">
-        <v>681.4413552903886</v>
+        <v>3753.865446064754</v>
       </c>
       <c r="D2" t="n">
-        <v>426.9445950726347</v>
+        <v>3301.043925363901</v>
       </c>
       <c r="E2" t="n">
-        <v>231.3682200462846</v>
+        <v>2666.5628586644</v>
       </c>
       <c r="F2" t="n">
-        <v>0</v>
+        <v>356.6099200932412</v>
       </c>
       <c r="G2" t="n">
-        <v>1008.522700216089</v>
+        <v>4257.919821064754</v>
       </c>
     </row>
     <row r="3">
@@ -1412,22 +1412,22 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>313.4639261599041</v>
+        <v>3307.685534485186</v>
       </c>
       <c r="C3" t="n">
-        <v>571.8430523530053</v>
+        <v>3753.865446064754</v>
       </c>
       <c r="D3" t="n">
-        <v>335.62382337891</v>
+        <v>3301.043925363901</v>
       </c>
       <c r="E3" t="n">
-        <v>168.155456557879</v>
+        <v>2666.5628586644</v>
       </c>
       <c r="F3" t="n">
-        <v>0</v>
+        <v>356.6099200932412</v>
       </c>
       <c r="G3" t="n">
-        <v>849.2864747954883</v>
+        <v>4257.919821064754</v>
       </c>
     </row>
     <row r="4">
@@ -1437,22 +1437,22 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>384.3064497379466</v>
+        <v>3307.685534485186</v>
       </c>
       <c r="C4" t="n">
-        <v>659.5216947029116</v>
+        <v>3753.865446064754</v>
       </c>
       <c r="D4" t="n">
-        <v>408.6804407338896</v>
+        <v>3301.043925363901</v>
       </c>
       <c r="E4" t="n">
-        <v>218.7256673486033</v>
+        <v>2666.5628586644</v>
       </c>
       <c r="F4" t="n">
-        <v>0</v>
+        <v>356.6099200932412</v>
       </c>
       <c r="G4" t="n">
-        <v>976.6754551319685</v>
+        <v>4257.919821064754</v>
       </c>
     </row>
     <row r="5">
@@ -1462,22 +1462,22 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>437.4383424214788</v>
+        <v>3390.773704422465</v>
       </c>
       <c r="C5" t="n">
-        <v>725.2806764653417</v>
+        <v>3845.795904326947</v>
       </c>
       <c r="D5" t="n">
-        <v>463.4729037501244</v>
+        <v>3383.444734899365</v>
       </c>
       <c r="E5" t="n">
-        <v>256.6533254416468</v>
+        <v>2735.001096414234</v>
       </c>
       <c r="F5" t="n">
-        <v>0</v>
+        <v>372.3839261986844</v>
       </c>
       <c r="G5" t="n">
-        <v>1072.217190384329</v>
+        <v>4362.194341826947</v>
       </c>
     </row>
     <row r="6">
@@ -1487,22 +1487,22 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>1075.021054623863</v>
+        <v>4055.479063920699</v>
       </c>
       <c r="C6" t="n">
-        <v>1514.388457614502</v>
+        <v>4581.239570424498</v>
       </c>
       <c r="D6" t="n">
-        <v>1120.982459944942</v>
+        <v>4042.65121118308</v>
       </c>
       <c r="E6" t="n">
-        <v>711.7852225581673</v>
+        <v>3282.506998412911</v>
       </c>
       <c r="F6" t="n">
-        <v>0</v>
+        <v>498.575975042232</v>
       </c>
       <c r="G6" t="n">
-        <v>2218.718013412655</v>
+        <v>5196.390507924498</v>
       </c>
     </row>
     <row r="7">
@@ -1512,47 +1512,47 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>313.4639261599041</v>
+        <v>3307.685534485186</v>
       </c>
       <c r="C7" t="n">
-        <v>571.8430523530053</v>
+        <v>3753.865446064754</v>
       </c>
       <c r="D7" t="n">
-        <v>335.62382337891</v>
+        <v>3301.043925363901</v>
       </c>
       <c r="E7" t="n">
-        <v>168.155456557879</v>
+        <v>2666.5628586644</v>
       </c>
       <c r="F7" t="n">
-        <v>0</v>
+        <v>356.6099200932412</v>
       </c>
       <c r="G7" t="n">
-        <v>849.2864747954883</v>
+        <v>4257.919821064754</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>Hedged (stochastic)</t>
+          <t>Stochastic commitment</t>
         </is>
       </c>
       <c r="B8" t="n">
-        <v>366.5958188434359</v>
+        <v>3307.685534485186</v>
       </c>
       <c r="C8" t="n">
-        <v>637.602034115435</v>
+        <v>3753.865446064754</v>
       </c>
       <c r="D8" t="n">
-        <v>390.4162863951446</v>
+        <v>3301.043925363901</v>
       </c>
       <c r="E8" t="n">
-        <v>206.0831146509223</v>
+        <v>2666.5628586644</v>
       </c>
       <c r="F8" t="n">
-        <v>0</v>
+        <v>356.6099200932412</v>
       </c>
       <c r="G8" t="n">
-        <v>944.8282100478484</v>
+        <v>4257.919821064754</v>
       </c>
     </row>
     <row r="10">
@@ -1743,79 +1743,79 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>0.6374999999999977</v>
+        <v>0.7306187500000004</v>
       </c>
       <c r="C2" t="n">
-        <v>0.6374999999999977</v>
+        <v>0.7306187500000004</v>
       </c>
       <c r="D2" t="n">
-        <v>0.6374999999999977</v>
+        <v>0.7306187500000004</v>
       </c>
       <c r="E2" t="n">
-        <v>0.6374999999999977</v>
+        <v>0.7306187500000004</v>
       </c>
       <c r="F2" t="n">
-        <v>0.6374999999999977</v>
+        <v>0.7306187500000004</v>
       </c>
       <c r="G2" t="n">
-        <v>0.6374999999999977</v>
+        <v>0.7306187500000004</v>
       </c>
       <c r="H2" t="n">
-        <v>0.6374999999999977</v>
+        <v>0.7306187500000004</v>
       </c>
       <c r="I2" t="n">
-        <v>0.6374999999999977</v>
+        <v>0.7306187500000004</v>
       </c>
       <c r="J2" t="n">
-        <v>0.6374999999999977</v>
+        <v>0.7306187500000004</v>
       </c>
       <c r="K2" t="n">
-        <v>0.6374999999999977</v>
+        <v>0.7306187500000004</v>
       </c>
       <c r="L2" t="n">
-        <v>0.6374999999999977</v>
+        <v>0.7306187500000004</v>
       </c>
       <c r="M2" t="n">
-        <v>0.6374999999999977</v>
+        <v>0.7306187500000004</v>
       </c>
       <c r="N2" t="n">
-        <v>0.6374999999999977</v>
+        <v>0.7306187500000004</v>
       </c>
       <c r="O2" t="n">
-        <v>0.6374999999999977</v>
+        <v>0.7306187500000004</v>
       </c>
       <c r="P2" t="n">
-        <v>0.6374999999999977</v>
+        <v>0.7306187500000004</v>
       </c>
       <c r="Q2" t="n">
-        <v>0.6374999999999977</v>
+        <v>0.7306187500000004</v>
       </c>
       <c r="R2" t="n">
-        <v>0.6374999999999977</v>
+        <v>0.7306187500000004</v>
       </c>
       <c r="S2" t="n">
-        <v>0.6374999999999977</v>
+        <v>0.7306187500000004</v>
       </c>
       <c r="T2" t="n">
-        <v>0.6374999999999977</v>
+        <v>0.7306187500000004</v>
       </c>
       <c r="U2" t="n">
-        <v>0.6374999999999977</v>
+        <v>0.7306187500000004</v>
       </c>
       <c r="V2" t="n">
-        <v>0.6374999999999977</v>
+        <v>0.7306187500000004</v>
       </c>
       <c r="W2" t="n">
-        <v>0.6374999999999977</v>
+        <v>0.7306187500000004</v>
       </c>
       <c r="X2" t="n">
-        <v>0.6374999999999977</v>
+        <v>0.7306187500000004</v>
       </c>
       <c r="Y2" t="n">
-        <v>0.6374999999999977</v>
+        <v>0.7306187500000004</v>
       </c>
       <c r="Z2" t="n">
-        <v>0.6374999999999977</v>
+        <v>0.7306187500000004</v>
       </c>
     </row>
     <row r="3">
@@ -1825,79 +1825,79 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>0.6687499999999976</v>
+        <v>0.7306187500000004</v>
       </c>
       <c r="C3" t="n">
-        <v>0.6687499999999976</v>
+        <v>0.7306187500000004</v>
       </c>
       <c r="D3" t="n">
-        <v>0.6687499999999976</v>
+        <v>0.7306187500000004</v>
       </c>
       <c r="E3" t="n">
-        <v>0.6687499999999976</v>
+        <v>0.7306187500000004</v>
       </c>
       <c r="F3" t="n">
-        <v>0.6687499999999976</v>
+        <v>0.7306187500000004</v>
       </c>
       <c r="G3" t="n">
-        <v>0.6687499999999976</v>
+        <v>0.7306187500000004</v>
       </c>
       <c r="H3" t="n">
-        <v>0.6687499999999976</v>
+        <v>0.7306187500000004</v>
       </c>
       <c r="I3" t="n">
-        <v>0.6687499999999976</v>
+        <v>0.7306187500000004</v>
       </c>
       <c r="J3" t="n">
-        <v>0.6687499999999976</v>
+        <v>0.7306187500000004</v>
       </c>
       <c r="K3" t="n">
-        <v>0.6687499999999976</v>
+        <v>0.7306187500000004</v>
       </c>
       <c r="L3" t="n">
-        <v>0.6687499999999976</v>
+        <v>0.7306187500000004</v>
       </c>
       <c r="M3" t="n">
-        <v>0.6687499999999976</v>
+        <v>0.7306187500000004</v>
       </c>
       <c r="N3" t="n">
-        <v>0.6687499999999976</v>
+        <v>0.7306187500000004</v>
       </c>
       <c r="O3" t="n">
-        <v>0.6687499999999976</v>
+        <v>0.7306187500000004</v>
       </c>
       <c r="P3" t="n">
-        <v>0.6687499999999976</v>
+        <v>0.7306187500000004</v>
       </c>
       <c r="Q3" t="n">
-        <v>0.6687499999999976</v>
+        <v>0.7306187500000004</v>
       </c>
       <c r="R3" t="n">
-        <v>0.6687499999999976</v>
+        <v>0.7306187500000004</v>
       </c>
       <c r="S3" t="n">
-        <v>0.6687499999999976</v>
+        <v>0.7306187500000004</v>
       </c>
       <c r="T3" t="n">
-        <v>0.6687499999999976</v>
+        <v>0.7306187500000004</v>
       </c>
       <c r="U3" t="n">
-        <v>0.6687499999999976</v>
+        <v>0.7306187500000004</v>
       </c>
       <c r="V3" t="n">
-        <v>0.6687499999999976</v>
+        <v>0.7306187500000004</v>
       </c>
       <c r="W3" t="n">
-        <v>0.6687499999999976</v>
+        <v>0.7306187500000004</v>
       </c>
       <c r="X3" t="n">
-        <v>0.6687499999999976</v>
+        <v>0.7306187500000004</v>
       </c>
       <c r="Y3" t="n">
-        <v>0.6687499999999976</v>
+        <v>0.7306187500000004</v>
       </c>
       <c r="Z3" t="n">
-        <v>0.6687499999999976</v>
+        <v>0.7306187500000004</v>
       </c>
     </row>
     <row r="4">
@@ -1907,79 +1907,79 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>0.6437499999999977</v>
+        <v>0.7306187500000004</v>
       </c>
       <c r="C4" t="n">
-        <v>0.6437499999999977</v>
+        <v>0.7306187500000004</v>
       </c>
       <c r="D4" t="n">
-        <v>0.6437499999999977</v>
+        <v>0.7306187500000004</v>
       </c>
       <c r="E4" t="n">
-        <v>0.6437499999999977</v>
+        <v>0.7306187500000004</v>
       </c>
       <c r="F4" t="n">
-        <v>0.6437499999999977</v>
+        <v>0.7306187500000004</v>
       </c>
       <c r="G4" t="n">
-        <v>0.6437499999999977</v>
+        <v>0.7306187500000004</v>
       </c>
       <c r="H4" t="n">
-        <v>0.6437499999999977</v>
+        <v>0.7306187500000004</v>
       </c>
       <c r="I4" t="n">
-        <v>0.6437499999999977</v>
+        <v>0.7306187500000004</v>
       </c>
       <c r="J4" t="n">
-        <v>0.6437499999999977</v>
+        <v>0.7306187500000004</v>
       </c>
       <c r="K4" t="n">
-        <v>0.6437499999999977</v>
+        <v>0.7306187500000004</v>
       </c>
       <c r="L4" t="n">
-        <v>0.6437499999999977</v>
+        <v>0.7306187500000004</v>
       </c>
       <c r="M4" t="n">
-        <v>0.6437499999999977</v>
+        <v>0.7306187500000004</v>
       </c>
       <c r="N4" t="n">
-        <v>0.6437499999999977</v>
+        <v>0.7306187500000004</v>
       </c>
       <c r="O4" t="n">
-        <v>0.6437499999999977</v>
+        <v>0.7306187500000004</v>
       </c>
       <c r="P4" t="n">
-        <v>0.6437499999999977</v>
+        <v>0.7306187500000004</v>
       </c>
       <c r="Q4" t="n">
-        <v>0.6437499999999977</v>
+        <v>0.7306187500000004</v>
       </c>
       <c r="R4" t="n">
-        <v>0.6437499999999977</v>
+        <v>0.7306187500000004</v>
       </c>
       <c r="S4" t="n">
-        <v>0.6437499999999977</v>
+        <v>0.7306187500000004</v>
       </c>
       <c r="T4" t="n">
-        <v>0.6437499999999977</v>
+        <v>0.7306187500000004</v>
       </c>
       <c r="U4" t="n">
-        <v>0.6437499999999977</v>
+        <v>0.7306187500000004</v>
       </c>
       <c r="V4" t="n">
-        <v>0.6437499999999977</v>
+        <v>0.7306187500000004</v>
       </c>
       <c r="W4" t="n">
-        <v>0.6437499999999977</v>
+        <v>0.7306187500000004</v>
       </c>
       <c r="X4" t="n">
-        <v>0.6437499999999977</v>
+        <v>0.7306187500000004</v>
       </c>
       <c r="Y4" t="n">
-        <v>0.6437499999999977</v>
+        <v>0.7306187500000004</v>
       </c>
       <c r="Z4" t="n">
-        <v>0.6437499999999977</v>
+        <v>0.7306187500000004</v>
       </c>
     </row>
     <row r="5">
@@ -1989,79 +1989,79 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>0.6249999999999978</v>
+        <v>0.7180218750000005</v>
       </c>
       <c r="C5" t="n">
-        <v>0.6249999999999978</v>
+        <v>0.7180218750000005</v>
       </c>
       <c r="D5" t="n">
-        <v>0.6249999999999978</v>
+        <v>0.7180218750000005</v>
       </c>
       <c r="E5" t="n">
-        <v>0.6249999999999978</v>
+        <v>0.7180218750000005</v>
       </c>
       <c r="F5" t="n">
-        <v>0.6249999999999978</v>
+        <v>0.7180218750000005</v>
       </c>
       <c r="G5" t="n">
-        <v>0.6249999999999978</v>
+        <v>0.7180218750000005</v>
       </c>
       <c r="H5" t="n">
-        <v>0.6249999999999978</v>
+        <v>0.7180218750000005</v>
       </c>
       <c r="I5" t="n">
-        <v>0.6249999999999978</v>
+        <v>0.7180218750000005</v>
       </c>
       <c r="J5" t="n">
-        <v>0.6249999999999978</v>
+        <v>0.7180218750000005</v>
       </c>
       <c r="K5" t="n">
-        <v>0.6249999999999978</v>
+        <v>0.7180218750000005</v>
       </c>
       <c r="L5" t="n">
-        <v>0.6249999999999978</v>
+        <v>0.7180218750000005</v>
       </c>
       <c r="M5" t="n">
-        <v>0.6249999999999978</v>
+        <v>0.7180218750000005</v>
       </c>
       <c r="N5" t="n">
-        <v>0.6249999999999978</v>
+        <v>0.7180218750000005</v>
       </c>
       <c r="O5" t="n">
-        <v>0.6249999999999978</v>
+        <v>0.7180218750000005</v>
       </c>
       <c r="P5" t="n">
-        <v>0.6249999999999978</v>
+        <v>0.7180218750000005</v>
       </c>
       <c r="Q5" t="n">
-        <v>0.6249999999999978</v>
+        <v>0.7180218750000005</v>
       </c>
       <c r="R5" t="n">
-        <v>0.6249999999999978</v>
+        <v>0.7180218750000005</v>
       </c>
       <c r="S5" t="n">
-        <v>0.6249999999999978</v>
+        <v>0.7180218750000005</v>
       </c>
       <c r="T5" t="n">
-        <v>0.6249999999999978</v>
+        <v>0.7180218750000005</v>
       </c>
       <c r="U5" t="n">
-        <v>0.6249999999999978</v>
+        <v>0.7180218750000005</v>
       </c>
       <c r="V5" t="n">
-        <v>0.6249999999999978</v>
+        <v>0.7180218750000005</v>
       </c>
       <c r="W5" t="n">
-        <v>0.6249999999999978</v>
+        <v>0.7180218750000005</v>
       </c>
       <c r="X5" t="n">
-        <v>0.6249999999999978</v>
+        <v>0.7180218750000005</v>
       </c>
       <c r="Y5" t="n">
-        <v>0.6249999999999978</v>
+        <v>0.7180218750000005</v>
       </c>
       <c r="Z5" t="n">
-        <v>0.6249999999999978</v>
+        <v>0.7180218750000004</v>
       </c>
     </row>
     <row r="6">
@@ -2071,79 +2071,79 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>0.4</v>
+        <v>0.6172468750000004</v>
       </c>
       <c r="C6" t="n">
-        <v>0.4</v>
+        <v>0.6172468750000004</v>
       </c>
       <c r="D6" t="n">
-        <v>0.4</v>
+        <v>0.6172468750000004</v>
       </c>
       <c r="E6" t="n">
-        <v>0.4</v>
+        <v>0.6172468750000004</v>
       </c>
       <c r="F6" t="n">
-        <v>0.4</v>
+        <v>0.6172468750000004</v>
       </c>
       <c r="G6" t="n">
-        <v>0.4</v>
+        <v>0.6172468750000004</v>
       </c>
       <c r="H6" t="n">
-        <v>0.4</v>
+        <v>0.6172468750000004</v>
       </c>
       <c r="I6" t="n">
-        <v>0.4</v>
+        <v>0.6172468750000004</v>
       </c>
       <c r="J6" t="n">
-        <v>0.4</v>
+        <v>0.6172468750000004</v>
       </c>
       <c r="K6" t="n">
-        <v>0.4</v>
+        <v>0.6172468750000004</v>
       </c>
       <c r="L6" t="n">
-        <v>0.4</v>
+        <v>0.6172468750000004</v>
       </c>
       <c r="M6" t="n">
-        <v>0.4</v>
+        <v>0.6172468750000004</v>
       </c>
       <c r="N6" t="n">
-        <v>0.4</v>
+        <v>0.6172468750000004</v>
       </c>
       <c r="O6" t="n">
-        <v>0.4</v>
+        <v>0.6172468750000004</v>
       </c>
       <c r="P6" t="n">
-        <v>0.4</v>
+        <v>0.6172468750000004</v>
       </c>
       <c r="Q6" t="n">
-        <v>0.4</v>
+        <v>0.6172468750000004</v>
       </c>
       <c r="R6" t="n">
-        <v>0.4</v>
+        <v>0.6172468750000004</v>
       </c>
       <c r="S6" t="n">
-        <v>0.4</v>
+        <v>0.6172468750000004</v>
       </c>
       <c r="T6" t="n">
-        <v>0.4</v>
+        <v>0.6172468750000004</v>
       </c>
       <c r="U6" t="n">
-        <v>0.4</v>
+        <v>0.6172468750000004</v>
       </c>
       <c r="V6" t="n">
-        <v>0.4</v>
+        <v>0.6172468750000004</v>
       </c>
       <c r="W6" t="n">
-        <v>0.4</v>
+        <v>0.6172468750000004</v>
       </c>
       <c r="X6" t="n">
-        <v>0.4</v>
+        <v>0.6172468750000004</v>
       </c>
       <c r="Y6" t="n">
-        <v>0.4</v>
+        <v>0.6172468750000004</v>
       </c>
       <c r="Z6" t="n">
-        <v>0.4000000000000001</v>
+        <v>0.6172468750000004</v>
       </c>
     </row>
     <row r="7">
@@ -2153,161 +2153,161 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>0.6687499999999976</v>
+        <v>0.7306187500000004</v>
       </c>
       <c r="C7" t="n">
-        <v>0.6687499999999976</v>
+        <v>0.7306187500000004</v>
       </c>
       <c r="D7" t="n">
-        <v>0.6687499999999976</v>
+        <v>0.7306187500000004</v>
       </c>
       <c r="E7" t="n">
-        <v>0.6687499999999976</v>
+        <v>0.7306187500000004</v>
       </c>
       <c r="F7" t="n">
-        <v>0.6687499999999976</v>
+        <v>0.7306187500000004</v>
       </c>
       <c r="G7" t="n">
-        <v>0.6687499999999976</v>
+        <v>0.7306187500000004</v>
       </c>
       <c r="H7" t="n">
-        <v>0.6687499999999976</v>
+        <v>0.7306187500000004</v>
       </c>
       <c r="I7" t="n">
-        <v>0.6687499999999976</v>
+        <v>0.7306187500000004</v>
       </c>
       <c r="J7" t="n">
-        <v>0.6687499999999976</v>
+        <v>0.7306187500000004</v>
       </c>
       <c r="K7" t="n">
-        <v>0.6687499999999976</v>
+        <v>0.7306187500000004</v>
       </c>
       <c r="L7" t="n">
-        <v>0.6687499999999976</v>
+        <v>0.7306187500000004</v>
       </c>
       <c r="M7" t="n">
-        <v>0.6687499999999976</v>
+        <v>0.7306187500000004</v>
       </c>
       <c r="N7" t="n">
-        <v>0.6687499999999976</v>
+        <v>0.7306187500000004</v>
       </c>
       <c r="O7" t="n">
-        <v>0.6687499999999976</v>
+        <v>0.7306187500000004</v>
       </c>
       <c r="P7" t="n">
-        <v>0.6687499999999976</v>
+        <v>0.7306187500000004</v>
       </c>
       <c r="Q7" t="n">
-        <v>0.6687499999999976</v>
+        <v>0.7306187500000004</v>
       </c>
       <c r="R7" t="n">
-        <v>0.6687499999999976</v>
+        <v>0.7306187500000004</v>
       </c>
       <c r="S7" t="n">
-        <v>0.6687499999999976</v>
+        <v>0.7306187500000004</v>
       </c>
       <c r="T7" t="n">
-        <v>0.6687499999999976</v>
+        <v>0.7306187500000004</v>
       </c>
       <c r="U7" t="n">
-        <v>0.6687499999999976</v>
+        <v>0.7306187500000004</v>
       </c>
       <c r="V7" t="n">
-        <v>0.6687499999999976</v>
+        <v>0.7306187500000004</v>
       </c>
       <c r="W7" t="n">
-        <v>0.6687499999999976</v>
+        <v>0.7306187500000004</v>
       </c>
       <c r="X7" t="n">
-        <v>0.6687499999999976</v>
+        <v>0.7306187500000004</v>
       </c>
       <c r="Y7" t="n">
-        <v>0.6687499999999976</v>
+        <v>0.7306187500000004</v>
       </c>
       <c r="Z7" t="n">
-        <v>0.6687499999999976</v>
+        <v>0.7306187500000004</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>Hedged (stochastic)</t>
+          <t>Stochastic commitment</t>
         </is>
       </c>
       <c r="B8" t="n">
-        <v>0.65</v>
+        <v>0.7306187499998338</v>
       </c>
       <c r="C8" t="n">
-        <v>0.65</v>
+        <v>0.7306187499998338</v>
       </c>
       <c r="D8" t="n">
-        <v>0.65</v>
+        <v>0.7306187499998338</v>
       </c>
       <c r="E8" t="n">
-        <v>0.65</v>
+        <v>0.7306187499998338</v>
       </c>
       <c r="F8" t="n">
-        <v>0.65</v>
+        <v>0.7306187499998338</v>
       </c>
       <c r="G8" t="n">
-        <v>0.65</v>
+        <v>0.7306187499998338</v>
       </c>
       <c r="H8" t="n">
-        <v>0.65</v>
+        <v>0.7306187499998338</v>
       </c>
       <c r="I8" t="n">
-        <v>0.65</v>
+        <v>0.7306187499998338</v>
       </c>
       <c r="J8" t="n">
-        <v>0.65</v>
+        <v>0.7306187499998338</v>
       </c>
       <c r="K8" t="n">
-        <v>0.65</v>
+        <v>0.7306187499998338</v>
       </c>
       <c r="L8" t="n">
-        <v>0.65</v>
+        <v>0.7306187499998338</v>
       </c>
       <c r="M8" t="n">
-        <v>0.65</v>
+        <v>0.7306187499998338</v>
       </c>
       <c r="N8" t="n">
-        <v>0.65</v>
+        <v>0.7306187499998338</v>
       </c>
       <c r="O8" t="n">
-        <v>0.65</v>
+        <v>0.7306187499998338</v>
       </c>
       <c r="P8" t="n">
-        <v>0.65</v>
+        <v>0.7306187499998338</v>
       </c>
       <c r="Q8" t="n">
-        <v>0.65</v>
+        <v>0.7306187499998338</v>
       </c>
       <c r="R8" t="n">
-        <v>0.65</v>
+        <v>0.7306187499998338</v>
       </c>
       <c r="S8" t="n">
-        <v>0.65</v>
+        <v>0.7306187499998338</v>
       </c>
       <c r="T8" t="n">
-        <v>0.65</v>
+        <v>0.7306187499998338</v>
       </c>
       <c r="U8" t="n">
-        <v>0.65</v>
+        <v>0.7306187499998338</v>
       </c>
       <c r="V8" t="n">
-        <v>0.65</v>
+        <v>0.7306187499998338</v>
       </c>
       <c r="W8" t="n">
-        <v>0.65</v>
+        <v>0.7306187499998338</v>
       </c>
       <c r="X8" t="n">
-        <v>0.65</v>
+        <v>0.7306187499998338</v>
       </c>
       <c r="Y8" t="n">
-        <v>0.65</v>
+        <v>0.7306187499998338</v>
       </c>
       <c r="Z8" t="n">
-        <v>0.65</v>
+        <v>0.7306187499998339</v>
       </c>
     </row>
   </sheetData>
@@ -2427,7 +2427,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>winter</t>
+          <t>summer</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
@@ -2441,40 +2441,40 @@
         </is>
       </c>
       <c r="D2" t="n">
-        <v>55.27734858696292</v>
+        <v>1675.735510873967</v>
       </c>
       <c r="E2" t="n">
         <v>0</v>
       </c>
       <c r="F2" t="n">
-        <v>256.2858889031916</v>
+        <v>2416.657070598648</v>
       </c>
       <c r="G2" t="n">
-        <v>201.0085403162287</v>
+        <v>740.9215597246817</v>
       </c>
       <c r="H2" t="n">
-        <v>461.1299155955714</v>
+        <v>2821.948510766032</v>
       </c>
       <c r="I2" t="n">
-        <v>402.0170806324575</v>
+        <v>3307.685534485186</v>
       </c>
       <c r="J2" t="n">
-        <v>2048.440266923798</v>
+        <v>1501.079408027346</v>
       </c>
       <c r="K2" t="n">
         <v>0</v>
       </c>
       <c r="L2" t="n">
-        <v>1806.484351240089</v>
+        <v>2160.29241836926</v>
       </c>
       <c r="M2" t="n">
-        <v>4256.941698796345</v>
+        <v>6969.057360881792</v>
       </c>
       <c r="N2" t="n">
-        <v>42.43620136378365</v>
+        <v>30.99834463259346</v>
       </c>
       <c r="O2" t="n">
-        <v>0.6375</v>
+        <v>0.73061875</v>
       </c>
       <c r="P2" t="inlineStr">
         <is>
@@ -2485,7 +2485,7 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>winter</t>
+          <t>summer</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
@@ -2499,40 +2499,40 @@
         </is>
       </c>
       <c r="D3" t="n">
-        <v>93.69818635242842</v>
+        <v>1901.778619953518</v>
       </c>
       <c r="E3" t="n">
-        <v>2.800328732141224</v>
+        <v>0</v>
       </c>
       <c r="F3" t="n">
-        <v>434.4188639976227</v>
+        <v>2742.644479872023</v>
       </c>
       <c r="G3" t="n">
-        <v>340.7206776451943</v>
+        <v>840.8658599185048</v>
       </c>
       <c r="H3" t="n">
-        <v>568.3883603559563</v>
+        <v>2965.394479872023</v>
       </c>
       <c r="I3" t="n">
-        <v>681.4413552903886</v>
+        <v>3753.865446064754</v>
       </c>
       <c r="J3" t="n">
-        <v>1339.694963583336</v>
+        <v>825</v>
       </c>
       <c r="K3" t="n">
         <v>0</v>
       </c>
       <c r="L3" t="n">
-        <v>2235.80537992262</v>
+        <v>2390.191914817039</v>
       </c>
       <c r="M3" t="n">
-        <v>4256.941698796345</v>
+        <v>6969.057360881792</v>
       </c>
       <c r="N3" t="n">
-        <v>52.52140005945576</v>
+        <v>34.29720536142364</v>
       </c>
       <c r="O3" t="n">
-        <v>0.6375</v>
+        <v>0.73061875</v>
       </c>
       <c r="P3" t="inlineStr">
         <is>
@@ -2543,7 +2543,7 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>winter</t>
+          <t>summer</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
@@ -2557,40 +2557,40 @@
         </is>
       </c>
       <c r="D4" t="n">
-        <v>58.70488182248729</v>
+        <v>1672.370747162953</v>
       </c>
       <c r="E4" t="n">
-        <v>0.04293153300938002</v>
+        <v>0</v>
       </c>
       <c r="F4" t="n">
-        <v>272.1771793588046</v>
+        <v>2411.804586444467</v>
       </c>
       <c r="G4" t="n">
-        <v>213.4722975363173</v>
+        <v>739.4338392815139</v>
       </c>
       <c r="H4" t="n">
-        <v>468.8825154759772</v>
+        <v>2823.714531095338</v>
       </c>
       <c r="I4" t="n">
-        <v>426.9445950726347</v>
+        <v>3301.043925363901</v>
       </c>
       <c r="J4" t="n">
-        <v>1967.053361171726</v>
+        <v>1525.592387595819</v>
       </c>
       <c r="K4" t="n">
         <v>0</v>
       </c>
       <c r="L4" t="n">
-        <v>1862.943742551984</v>
+        <v>2142.421047922072</v>
       </c>
       <c r="M4" t="n">
-        <v>4256.941698796345</v>
+        <v>6969.057360881792</v>
       </c>
       <c r="N4" t="n">
-        <v>43.76249134628114</v>
+        <v>30.74190578409864</v>
       </c>
       <c r="O4" t="n">
-        <v>0.6375</v>
+        <v>0.73061875</v>
       </c>
       <c r="P4" t="inlineStr">
         <is>
@@ -2601,7 +2601,7 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>winter</t>
+          <t>summer</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
@@ -2615,40 +2615,40 @@
         </is>
       </c>
       <c r="D5" t="n">
-        <v>31.81313025636415</v>
+        <v>1350.930742252985</v>
       </c>
       <c r="E5" t="n">
-        <v>0.2685354238417261</v>
+        <v>0.2196275246308232</v>
       </c>
       <c r="F5" t="n">
-        <v>147.4972402795064</v>
+        <v>1948.240822593811</v>
       </c>
       <c r="G5" t="n">
-        <v>115.6841100231423</v>
+        <v>597.3100803408257</v>
       </c>
       <c r="H5" t="n">
-        <v>421.1005506381649</v>
+        <v>2629.477909188668</v>
       </c>
       <c r="I5" t="n">
-        <v>231.3682200462846</v>
+        <v>2666.5628586644</v>
       </c>
       <c r="J5" t="n">
-        <v>2736.033103586585</v>
+        <v>2523.100320721695</v>
       </c>
       <c r="K5" t="n">
         <v>0</v>
       </c>
       <c r="L5" t="n">
-        <v>1289.540375163475</v>
+        <v>1779.394181495698</v>
       </c>
       <c r="M5" t="n">
-        <v>4256.941698796345</v>
+        <v>6969.057360881792</v>
       </c>
       <c r="N5" t="n">
-        <v>30.29264825327755</v>
+        <v>25.53278139858145</v>
       </c>
       <c r="O5" t="n">
-        <v>0.6375</v>
+        <v>0.73061875</v>
       </c>
       <c r="P5" t="inlineStr">
         <is>
@@ -2659,7 +2659,7 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>winter</t>
+          <t>summer</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
@@ -2673,40 +2673,40 @@
         </is>
       </c>
       <c r="D6" t="n">
-        <v>0</v>
+        <v>180.6652719552377</v>
       </c>
       <c r="E6" t="n">
-        <v>0</v>
+        <v>15.39817218019797</v>
       </c>
       <c r="F6" t="n">
-        <v>0</v>
+        <v>260.5458940561238</v>
       </c>
       <c r="G6" t="n">
-        <v>0</v>
+        <v>79.88062210088603</v>
       </c>
       <c r="H6" t="n">
-        <v>425.6941698796345</v>
+        <v>1935.17318020882</v>
       </c>
       <c r="I6" t="n">
-        <v>0</v>
+        <v>356.6099200932412</v>
       </c>
       <c r="J6" t="n">
-        <v>4256.941698796345</v>
+        <v>6202.323282047022</v>
       </c>
       <c r="K6" t="n">
         <v>0</v>
       </c>
       <c r="L6" t="n">
-        <v>0</v>
+        <v>410.1241587415291</v>
       </c>
       <c r="M6" t="n">
-        <v>4256.941698796345</v>
+        <v>6969.057360881792</v>
       </c>
       <c r="N6" t="n">
-        <v>0</v>
+        <v>5.884930163491096</v>
       </c>
       <c r="O6" t="n">
-        <v>0.6375</v>
+        <v>0.73061875</v>
       </c>
       <c r="P6" t="inlineStr">
         <is>
@@ -2717,7 +2717,7 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>winter</t>
+          <t>summer</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
@@ -2731,22 +2731,22 @@
         </is>
       </c>
       <c r="D7" t="n">
-        <v>138.6718712797123</v>
+        <v>2157.142017348049</v>
       </c>
       <c r="E7" t="n">
-        <v>4.645221342026389</v>
+        <v>0</v>
       </c>
       <c r="F7" t="n">
-        <v>642.9332213877567</v>
+        <v>3110.916057266554</v>
       </c>
       <c r="G7" t="n">
-        <v>504.2613501080444</v>
+        <v>953.7740399185049</v>
       </c>
       <c r="H7" t="n">
-        <v>642.9332213877567</v>
+        <v>3110.916057266554</v>
       </c>
       <c r="I7" t="n">
-        <v>1008.522700216089</v>
+        <v>4257.919821064754</v>
       </c>
       <c r="J7" t="n">
         <v>0</v>
@@ -2755,16 +2755,16 @@
         <v>0</v>
       </c>
       <c r="L7" t="n">
-        <v>3248.418998580256</v>
+        <v>2711.137539817038</v>
       </c>
       <c r="M7" t="n">
-        <v>4256.941698796345</v>
+        <v>6969.057360881792</v>
       </c>
       <c r="N7" t="n">
-        <v>76.30875</v>
+        <v>38.90249999999999</v>
       </c>
       <c r="O7" t="n">
-        <v>0.6375</v>
+        <v>0.73061875</v>
       </c>
       <c r="P7" t="inlineStr">
         <is>
@@ -2775,7 +2775,7 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>winter</t>
+          <t>summer</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
@@ -2789,40 +2789,40 @@
         </is>
       </c>
       <c r="D8" t="n">
-        <v>52.89703753948382</v>
+        <v>1675.735510873967</v>
       </c>
       <c r="E8" t="n">
-        <v>2.380311047479097</v>
+        <v>0</v>
       </c>
       <c r="F8" t="n">
-        <v>209.6290006194359</v>
+        <v>2416.657070598648</v>
       </c>
       <c r="G8" t="n">
-        <v>156.731963079952</v>
+        <v>740.9215597246817</v>
       </c>
       <c r="H8" t="n">
-        <v>414.4730273118157</v>
+        <v>2821.948510766032</v>
       </c>
       <c r="I8" t="n">
-        <v>313.4639261599041</v>
+        <v>3307.685534485186</v>
       </c>
       <c r="J8" t="n">
-        <v>2048.440266923798</v>
+        <v>1501.079408027346</v>
       </c>
       <c r="K8" t="n">
         <v>0</v>
       </c>
       <c r="L8" t="n">
-        <v>1895.037505712643</v>
+        <v>2160.29241836926</v>
       </c>
       <c r="M8" t="n">
-        <v>4256.941698796345</v>
+        <v>6969.057360881792</v>
       </c>
       <c r="N8" t="n">
-        <v>44.51640731298873</v>
+        <v>30.99834463259346</v>
       </c>
       <c r="O8" t="n">
-        <v>0.6687499999999998</v>
+        <v>0.73061875</v>
       </c>
       <c r="P8" t="inlineStr">
         <is>
@@ -2833,7 +2833,7 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>winter</t>
+          <t>summer</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
@@ -2847,40 +2847,40 @@
         </is>
       </c>
       <c r="D9" t="n">
-        <v>96.49851508456965</v>
+        <v>1901.778619953518</v>
       </c>
       <c r="E9" t="n">
         <v>0</v>
       </c>
       <c r="F9" t="n">
-        <v>382.4200412610722</v>
+        <v>2742.644479872023</v>
       </c>
       <c r="G9" t="n">
-        <v>285.9215261765026</v>
+        <v>840.8658599185048</v>
       </c>
       <c r="H9" t="n">
-        <v>516.3895376194058</v>
+        <v>2965.394479872023</v>
       </c>
       <c r="I9" t="n">
-        <v>571.8430523530053</v>
+        <v>3753.865446064754</v>
       </c>
       <c r="J9" t="n">
-        <v>1339.694963583336</v>
+        <v>825</v>
       </c>
       <c r="K9" t="n">
         <v>0</v>
       </c>
       <c r="L9" t="n">
-        <v>2345.403682860004</v>
+        <v>2390.191914817039</v>
       </c>
       <c r="M9" t="n">
-        <v>4256.941698796345</v>
+        <v>6969.057360881792</v>
       </c>
       <c r="N9" t="n">
-        <v>55.09597849374281</v>
+        <v>34.29720536142364</v>
       </c>
       <c r="O9" t="n">
-        <v>0.6687499999999998</v>
+        <v>0.73061875</v>
       </c>
       <c r="P9" t="inlineStr">
         <is>
@@ -2891,7 +2891,7 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>winter</t>
+          <t>summer</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
@@ -2905,40 +2905,40 @@
         </is>
       </c>
       <c r="D10" t="n">
-        <v>56.63652019519108</v>
+        <v>1672.370747162953</v>
       </c>
       <c r="E10" t="n">
-        <v>2.111293160305593</v>
+        <v>0</v>
       </c>
       <c r="F10" t="n">
-        <v>224.4484318846461</v>
+        <v>2411.804586444467</v>
       </c>
       <c r="G10" t="n">
-        <v>167.811911689455</v>
+        <v>739.4338392815139</v>
       </c>
       <c r="H10" t="n">
-        <v>421.1537680018187</v>
+        <v>2823.714531095338</v>
       </c>
       <c r="I10" t="n">
-        <v>335.62382337891</v>
+        <v>3301.043925363901</v>
       </c>
       <c r="J10" t="n">
-        <v>1967.053361171726</v>
+        <v>1525.592387595819</v>
       </c>
       <c r="K10" t="n">
         <v>0</v>
       </c>
       <c r="L10" t="n">
-        <v>1954.264514245709</v>
+        <v>2142.421047922072</v>
       </c>
       <c r="M10" t="n">
-        <v>4256.941698796345</v>
+        <v>6969.057360881792</v>
       </c>
       <c r="N10" t="n">
-        <v>45.90771151031453</v>
+        <v>30.74190578409864</v>
       </c>
       <c r="O10" t="n">
-        <v>0.6687499999999998</v>
+        <v>0.73061875</v>
       </c>
       <c r="P10" t="inlineStr">
         <is>
@@ -2949,7 +2949,7 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>winter</t>
+          <t>summer</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
@@ -2963,40 +2963,40 @@
         </is>
       </c>
       <c r="D11" t="n">
-        <v>28.3762332941421</v>
+        <v>1350.930742252985</v>
       </c>
       <c r="E11" t="n">
-        <v>3.705432386063777</v>
+        <v>0.2196275246308232</v>
       </c>
       <c r="F11" t="n">
-        <v>112.4539615730816</v>
+        <v>1948.240822593811</v>
       </c>
       <c r="G11" t="n">
-        <v>84.07772827893949</v>
+        <v>597.3100803408257</v>
       </c>
       <c r="H11" t="n">
-        <v>386.0572719317401</v>
+        <v>2629.477909188668</v>
       </c>
       <c r="I11" t="n">
-        <v>168.155456557879</v>
+        <v>2666.5628586644</v>
       </c>
       <c r="J11" t="n">
-        <v>2736.033103586585</v>
+        <v>2523.100320721695</v>
       </c>
       <c r="K11" t="n">
         <v>0</v>
       </c>
       <c r="L11" t="n">
-        <v>1352.75313865188</v>
+        <v>1779.394181495698</v>
       </c>
       <c r="M11" t="n">
-        <v>4256.941698796345</v>
+        <v>6969.057360881792</v>
       </c>
       <c r="N11" t="n">
-        <v>31.77758199118331</v>
+        <v>25.53278139858145</v>
       </c>
       <c r="O11" t="n">
-        <v>0.6687499999999998</v>
+        <v>0.73061875</v>
       </c>
       <c r="P11" t="inlineStr">
         <is>
@@ -3007,7 +3007,7 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>winter</t>
+          <t>summer</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
@@ -3021,40 +3021,40 @@
         </is>
       </c>
       <c r="D12" t="n">
-        <v>0</v>
+        <v>180.6652719552377</v>
       </c>
       <c r="E12" t="n">
-        <v>0</v>
+        <v>15.39817218019797</v>
       </c>
       <c r="F12" t="n">
-        <v>0</v>
+        <v>260.5458940561238</v>
       </c>
       <c r="G12" t="n">
-        <v>0</v>
+        <v>79.88062210088603</v>
       </c>
       <c r="H12" t="n">
-        <v>425.6941698796345</v>
+        <v>1935.17318020882</v>
       </c>
       <c r="I12" t="n">
-        <v>0</v>
+        <v>356.6099200932412</v>
       </c>
       <c r="J12" t="n">
-        <v>4256.941698796345</v>
+        <v>6202.323282047022</v>
       </c>
       <c r="K12" t="n">
         <v>0</v>
       </c>
       <c r="L12" t="n">
-        <v>0</v>
+        <v>410.1241587415291</v>
       </c>
       <c r="M12" t="n">
-        <v>4256.941698796345</v>
+        <v>6969.057360881792</v>
       </c>
       <c r="N12" t="n">
-        <v>0</v>
+        <v>5.884930163491096</v>
       </c>
       <c r="O12" t="n">
-        <v>0.6687499999999998</v>
+        <v>0.73061875</v>
       </c>
       <c r="P12" t="inlineStr">
         <is>
@@ -3065,7 +3065,7 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>winter</t>
+          <t>summer</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
@@ -3079,22 +3079,22 @@
         </is>
       </c>
       <c r="D13" t="n">
-        <v>143.3170926217387</v>
+        <v>2157.142017348049</v>
       </c>
       <c r="E13" t="n">
         <v>0</v>
       </c>
       <c r="F13" t="n">
-        <v>567.9603300194827</v>
+        <v>3110.916057266554</v>
       </c>
       <c r="G13" t="n">
-        <v>424.6432373977441</v>
+        <v>953.7740399185049</v>
       </c>
       <c r="H13" t="n">
-        <v>567.9603300194827</v>
+        <v>3110.916057266554</v>
       </c>
       <c r="I13" t="n">
-        <v>849.2864747954883</v>
+        <v>4257.919821064754</v>
       </c>
       <c r="J13" t="n">
         <v>0</v>
@@ -3103,16 +3103,16 @@
         <v>0</v>
       </c>
       <c r="L13" t="n">
-        <v>3407.655224000856</v>
+        <v>2711.137539817038</v>
       </c>
       <c r="M13" t="n">
-        <v>4256.941698796345</v>
+        <v>6969.057360881792</v>
       </c>
       <c r="N13" t="n">
-        <v>80.049375</v>
+        <v>38.90249999999999</v>
       </c>
       <c r="O13" t="n">
-        <v>0.6687499999999998</v>
+        <v>0.73061875</v>
       </c>
       <c r="P13" t="inlineStr">
         <is>
@@ -3123,7 +3123,7 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>winter</t>
+          <t>summer</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
@@ -3137,40 +3137,40 @@
         </is>
       </c>
       <c r="D14" t="n">
-        <v>55.24405214982986</v>
+        <v>1675.735510873967</v>
       </c>
       <c r="E14" t="n">
-        <v>0.03329643713306041</v>
+        <v>0</v>
       </c>
       <c r="F14" t="n">
-        <v>247.3972770188031</v>
+        <v>2416.657070598648</v>
       </c>
       <c r="G14" t="n">
-        <v>192.1532248689733</v>
+        <v>740.9215597246817</v>
       </c>
       <c r="H14" t="n">
-        <v>452.2413037111829</v>
+        <v>2821.948510766032</v>
       </c>
       <c r="I14" t="n">
-        <v>384.3064497379466</v>
+        <v>3307.685534485186</v>
       </c>
       <c r="J14" t="n">
-        <v>2048.440266923798</v>
+        <v>1501.079408027346</v>
       </c>
       <c r="K14" t="n">
         <v>0</v>
       </c>
       <c r="L14" t="n">
-        <v>1824.1949821346</v>
+        <v>2160.29241836926</v>
       </c>
       <c r="M14" t="n">
-        <v>4256.941698796345</v>
+        <v>6969.057360881792</v>
       </c>
       <c r="N14" t="n">
-        <v>42.85224255362467</v>
+        <v>30.99834463259346</v>
       </c>
       <c r="O14" t="n">
-        <v>0.64375</v>
+        <v>0.73061875</v>
       </c>
       <c r="P14" t="inlineStr">
         <is>
@@ -3181,7 +3181,7 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>winter</t>
+          <t>summer</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
@@ -3195,40 +3195,40 @@
         </is>
       </c>
       <c r="D15" t="n">
-        <v>94.80624361354364</v>
+        <v>1901.778619953518</v>
       </c>
       <c r="E15" t="n">
-        <v>1.692271471026004</v>
+        <v>0</v>
       </c>
       <c r="F15" t="n">
-        <v>424.5670909649994</v>
+        <v>2742.644479872023</v>
       </c>
       <c r="G15" t="n">
-        <v>329.7608473514558</v>
+        <v>840.8658599185048</v>
       </c>
       <c r="H15" t="n">
-        <v>558.5365873233329</v>
+        <v>2965.394479872023</v>
       </c>
       <c r="I15" t="n">
-        <v>659.5216947029116</v>
+        <v>3753.865446064754</v>
       </c>
       <c r="J15" t="n">
-        <v>1339.694963583336</v>
+        <v>825</v>
       </c>
       <c r="K15" t="n">
         <v>0</v>
       </c>
       <c r="L15" t="n">
-        <v>2257.725040510098</v>
+        <v>2390.191914817039</v>
       </c>
       <c r="M15" t="n">
-        <v>4256.941698796345</v>
+        <v>6969.057360881792</v>
       </c>
       <c r="N15" t="n">
-        <v>53.03631574631318</v>
+        <v>34.29720536142364</v>
       </c>
       <c r="O15" t="n">
-        <v>0.64375</v>
+        <v>0.73061875</v>
       </c>
       <c r="P15" t="inlineStr">
         <is>
@@ -3239,7 +3239,7 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>winter</t>
+          <t>summer</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
@@ -3253,40 +3253,40 @@
         </is>
       </c>
       <c r="D16" t="n">
-        <v>58.74781335549667</v>
+        <v>1672.370747162953</v>
       </c>
       <c r="E16" t="n">
         <v>0</v>
       </c>
       <c r="F16" t="n">
-        <v>263.0880337224414</v>
+        <v>2411.804586444467</v>
       </c>
       <c r="G16" t="n">
-        <v>204.3402203669447</v>
+        <v>739.4338392815139</v>
       </c>
       <c r="H16" t="n">
-        <v>459.7933698396141</v>
+        <v>2823.714531095338</v>
       </c>
       <c r="I16" t="n">
-        <v>408.6804407338896</v>
+        <v>3301.043925363901</v>
       </c>
       <c r="J16" t="n">
-        <v>1967.053361171726</v>
+        <v>1525.592387595819</v>
       </c>
       <c r="K16" t="n">
         <v>0</v>
       </c>
       <c r="L16" t="n">
-        <v>1881.207896890729</v>
+        <v>2142.421047922072</v>
       </c>
       <c r="M16" t="n">
-        <v>4256.941698796345</v>
+        <v>6969.057360881792</v>
       </c>
       <c r="N16" t="n">
-        <v>44.19153537908782</v>
+        <v>30.74190578409864</v>
       </c>
       <c r="O16" t="n">
-        <v>0.64375</v>
+        <v>0.73061875</v>
       </c>
       <c r="P16" t="inlineStr">
         <is>
@@ -3297,7 +3297,7 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>winter</t>
+          <t>summer</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
@@ -3311,40 +3311,40 @@
         </is>
       </c>
       <c r="D17" t="n">
-        <v>31.44181468136175</v>
+        <v>1350.930742252985</v>
       </c>
       <c r="E17" t="n">
-        <v>0.6398509988441248</v>
+        <v>0.2196275246308232</v>
       </c>
       <c r="F17" t="n">
-        <v>140.8046483556634</v>
+        <v>1948.240822593811</v>
       </c>
       <c r="G17" t="n">
-        <v>109.3628336743017</v>
+        <v>597.3100803408257</v>
       </c>
       <c r="H17" t="n">
-        <v>414.4079587143219</v>
+        <v>2629.477909188668</v>
       </c>
       <c r="I17" t="n">
-        <v>218.7256673486033</v>
+        <v>2666.5628586644</v>
       </c>
       <c r="J17" t="n">
-        <v>2736.033103586585</v>
+        <v>2523.100320721695</v>
       </c>
       <c r="K17" t="n">
         <v>0</v>
       </c>
       <c r="L17" t="n">
-        <v>1302.182927861156</v>
+        <v>1779.394181495698</v>
       </c>
       <c r="M17" t="n">
-        <v>4256.941698796345</v>
+        <v>6969.057360881792</v>
       </c>
       <c r="N17" t="n">
-        <v>30.58963500085871</v>
+        <v>25.53278139858145</v>
       </c>
       <c r="O17" t="n">
-        <v>0.64375</v>
+        <v>0.73061875</v>
       </c>
       <c r="P17" t="inlineStr">
         <is>
@@ -3355,7 +3355,7 @@
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>winter</t>
+          <t>summer</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
@@ -3369,40 +3369,40 @@
         </is>
       </c>
       <c r="D18" t="n">
-        <v>0</v>
+        <v>180.6652719552377</v>
       </c>
       <c r="E18" t="n">
-        <v>0</v>
+        <v>15.39817218019797</v>
       </c>
       <c r="F18" t="n">
-        <v>0</v>
+        <v>260.5458940561238</v>
       </c>
       <c r="G18" t="n">
-        <v>0</v>
+        <v>79.88062210088603</v>
       </c>
       <c r="H18" t="n">
-        <v>425.6941698796345</v>
+        <v>1935.17318020882</v>
       </c>
       <c r="I18" t="n">
-        <v>0</v>
+        <v>356.6099200932412</v>
       </c>
       <c r="J18" t="n">
-        <v>4256.941698796345</v>
+        <v>6202.323282047022</v>
       </c>
       <c r="K18" t="n">
         <v>0</v>
       </c>
       <c r="L18" t="n">
-        <v>0</v>
+        <v>410.1241587415291</v>
       </c>
       <c r="M18" t="n">
-        <v>4256.941698796345</v>
+        <v>6969.057360881792</v>
       </c>
       <c r="N18" t="n">
-        <v>0</v>
+        <v>5.884930163491096</v>
       </c>
       <c r="O18" t="n">
-        <v>0.64375</v>
+        <v>0.73061875</v>
       </c>
       <c r="P18" t="inlineStr">
         <is>
@@ -3413,7 +3413,7 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>winter</t>
+          <t>summer</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
@@ -3427,22 +3427,22 @@
         </is>
       </c>
       <c r="D19" t="n">
-        <v>140.3970966752207</v>
+        <v>2157.142017348049</v>
       </c>
       <c r="E19" t="n">
-        <v>2.919995946517986</v>
+        <v>0</v>
       </c>
       <c r="F19" t="n">
-        <v>628.7348242412048</v>
+        <v>3110.916057266554</v>
       </c>
       <c r="G19" t="n">
-        <v>488.3377275659842</v>
+        <v>953.7740399185049</v>
       </c>
       <c r="H19" t="n">
-        <v>628.7348242412048</v>
+        <v>3110.916057266554</v>
       </c>
       <c r="I19" t="n">
-        <v>976.6754551319685</v>
+        <v>4257.919821064754</v>
       </c>
       <c r="J19" t="n">
         <v>0</v>
@@ -3451,16 +3451,16 @@
         <v>0</v>
       </c>
       <c r="L19" t="n">
-        <v>3280.266243664376</v>
+        <v>2711.137539817038</v>
       </c>
       <c r="M19" t="n">
-        <v>4256.941698796345</v>
+        <v>6969.057360881792</v>
       </c>
       <c r="N19" t="n">
-        <v>77.05687500000001</v>
+        <v>38.90249999999999</v>
       </c>
       <c r="O19" t="n">
-        <v>0.64375</v>
+        <v>0.73061875</v>
       </c>
       <c r="P19" t="inlineStr">
         <is>
@@ -3471,7 +3471,7 @@
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>winter</t>
+          <t>summer</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
@@ -3485,40 +3485,40 @@
         </is>
       </c>
       <c r="D20" t="n">
-        <v>54.67979280268491</v>
+        <v>1675.116383159482</v>
       </c>
       <c r="E20" t="n">
-        <v>0.5975557842780006</v>
+        <v>0.6191277144848755</v>
       </c>
       <c r="F20" t="n">
-        <v>273.3989640134242</v>
+        <v>2434.649692950114</v>
       </c>
       <c r="G20" t="n">
-        <v>218.7191712107393</v>
+        <v>759.5333097906323</v>
       </c>
       <c r="H20" t="n">
-        <v>478.242990705804</v>
+        <v>2839.941133117497</v>
       </c>
       <c r="I20" t="n">
-        <v>437.4383424214788</v>
+        <v>3390.773704422465</v>
       </c>
       <c r="J20" t="n">
-        <v>2048.440266923798</v>
+        <v>1501.079408027346</v>
       </c>
       <c r="K20" t="n">
         <v>0</v>
       </c>
       <c r="L20" t="n">
-        <v>1771.063089451068</v>
+        <v>2077.204248431981</v>
       </c>
       <c r="M20" t="n">
-        <v>4256.941698796345</v>
+        <v>6969.057360881792</v>
       </c>
       <c r="N20" t="n">
-        <v>41.60411898410162</v>
+        <v>29.80610060826294</v>
       </c>
       <c r="O20" t="n">
-        <v>0.625</v>
+        <v>0.7180218750000001</v>
       </c>
       <c r="P20" t="inlineStr">
         <is>
@@ -3529,7 +3529,7 @@
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>winter</t>
+          <t>summer</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
@@ -3543,40 +3543,40 @@
         </is>
       </c>
       <c r="D21" t="n">
-        <v>90.66008455816774</v>
+        <v>1899.907303522919</v>
       </c>
       <c r="E21" t="n">
-        <v>5.838430526401908</v>
+        <v>1.871316430598654</v>
       </c>
       <c r="F21" t="n">
-        <v>453.3004227908386</v>
+        <v>2761.365586092155</v>
       </c>
       <c r="G21" t="n">
-        <v>362.6403382326708</v>
+        <v>861.4582825692362</v>
       </c>
       <c r="H21" t="n">
-        <v>587.2699191491722</v>
+        <v>2984.115586092155</v>
       </c>
       <c r="I21" t="n">
-        <v>725.2806764653417</v>
+        <v>3845.795904326947</v>
       </c>
       <c r="J21" t="n">
-        <v>1339.694963583336</v>
+        <v>825</v>
       </c>
       <c r="K21" t="n">
         <v>0</v>
       </c>
       <c r="L21" t="n">
-        <v>2191.966058747667</v>
+        <v>2298.261456554845</v>
       </c>
       <c r="M21" t="n">
-        <v>4256.941698796345</v>
+        <v>6969.057360881792</v>
       </c>
       <c r="N21" t="n">
-        <v>51.49156868574094</v>
+        <v>32.97808207829196</v>
       </c>
       <c r="O21" t="n">
-        <v>0.625</v>
+        <v>0.7180218750000001</v>
       </c>
       <c r="P21" t="inlineStr">
         <is>
@@ -3587,7 +3587,7 @@
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>winter</t>
+          <t>summer</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
@@ -3601,40 +3601,40 @@
         </is>
       </c>
       <c r="D22" t="n">
-        <v>57.93411296876559</v>
+        <v>1671.495711893862</v>
       </c>
       <c r="E22" t="n">
-        <v>0.8137003867310852</v>
+        <v>0.8750352690906311</v>
       </c>
       <c r="F22" t="n">
-        <v>289.6705648438278</v>
+        <v>2429.38733251132</v>
       </c>
       <c r="G22" t="n">
-        <v>231.7364518750622</v>
+        <v>757.8916206174579</v>
       </c>
       <c r="H22" t="n">
-        <v>486.3759009610004</v>
+        <v>2841.297277162191</v>
       </c>
       <c r="I22" t="n">
-        <v>463.4729037501244</v>
+        <v>3383.444734899365</v>
       </c>
       <c r="J22" t="n">
-        <v>1967.053361171726</v>
+        <v>1525.592387595819</v>
       </c>
       <c r="K22" t="n">
         <v>0</v>
       </c>
       <c r="L22" t="n">
-        <v>1826.415433874494</v>
+        <v>2060.020238386608</v>
       </c>
       <c r="M22" t="n">
-        <v>4256.941698796345</v>
+        <v>6969.057360881792</v>
       </c>
       <c r="N22" t="n">
-        <v>42.90440328066779</v>
+        <v>29.55952479240255</v>
       </c>
       <c r="O22" t="n">
-        <v>0.625</v>
+        <v>0.7180218750000001</v>
       </c>
       <c r="P22" t="inlineStr">
         <is>
@@ -3645,7 +3645,7 @@
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>winter</t>
+          <t>summer</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
@@ -3659,40 +3659,40 @@
         </is>
       </c>
       <c r="D23" t="n">
-        <v>32.08166568020587</v>
+        <v>1351.150369777616</v>
       </c>
       <c r="E23" t="n">
         <v>0</v>
       </c>
       <c r="F23" t="n">
-        <v>160.4083284010293</v>
+        <v>1963.790615374405</v>
       </c>
       <c r="G23" t="n">
-        <v>128.3266627208234</v>
+        <v>612.6402455967886</v>
       </c>
       <c r="H23" t="n">
-        <v>434.0116387596878</v>
+        <v>2645.027701969262</v>
       </c>
       <c r="I23" t="n">
-        <v>256.6533254416468</v>
+        <v>2735.001096414234</v>
       </c>
       <c r="J23" t="n">
-        <v>2736.033103586585</v>
+        <v>2523.100320721695</v>
       </c>
       <c r="K23" t="n">
         <v>0</v>
       </c>
       <c r="L23" t="n">
-        <v>1264.255269768113</v>
+        <v>1710.955943745863</v>
       </c>
       <c r="M23" t="n">
-        <v>4256.941698796345</v>
+        <v>6969.057360881792</v>
       </c>
       <c r="N23" t="n">
-        <v>29.69867475811525</v>
+        <v>24.55075134478986</v>
       </c>
       <c r="O23" t="n">
-        <v>0.625</v>
+        <v>0.7180218750000001</v>
       </c>
       <c r="P23" t="inlineStr">
         <is>
@@ -3703,7 +3703,7 @@
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>winter</t>
+          <t>summer</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
@@ -3717,40 +3717,40 @@
         </is>
       </c>
       <c r="D24" t="n">
-        <v>0</v>
+        <v>183.9658054405357</v>
       </c>
       <c r="E24" t="n">
-        <v>0</v>
+        <v>12.09763869490001</v>
       </c>
       <c r="F24" t="n">
-        <v>0</v>
+        <v>267.379804909041</v>
       </c>
       <c r="G24" t="n">
-        <v>0</v>
+        <v>83.41399946850531</v>
       </c>
       <c r="H24" t="n">
-        <v>425.6941698796345</v>
+        <v>1942.007091061737</v>
       </c>
       <c r="I24" t="n">
-        <v>0</v>
+        <v>372.3839261986844</v>
       </c>
       <c r="J24" t="n">
-        <v>4256.941698796345</v>
+        <v>6202.323282047022</v>
       </c>
       <c r="K24" t="n">
         <v>0</v>
       </c>
       <c r="L24" t="n">
-        <v>0</v>
+        <v>394.3501526360857</v>
       </c>
       <c r="M24" t="n">
-        <v>4256.941698796345</v>
+        <v>6969.057360881792</v>
       </c>
       <c r="N24" t="n">
-        <v>0</v>
+        <v>5.658586695664517</v>
       </c>
       <c r="O24" t="n">
-        <v>0.625</v>
+        <v>0.7180218750000001</v>
       </c>
       <c r="P24" t="inlineStr">
         <is>
@@ -3761,7 +3761,7 @@
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>winter</t>
+          <t>summer</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
@@ -3775,22 +3775,22 @@
         </is>
       </c>
       <c r="D25" t="n">
-        <v>134.0271487980411</v>
+        <v>2155.019427863739</v>
       </c>
       <c r="E25" t="n">
-        <v>9.289943823697513</v>
+        <v>2.122589484309628</v>
       </c>
       <c r="F25" t="n">
-        <v>670.1357439902057</v>
+        <v>3132.150960432975</v>
       </c>
       <c r="G25" t="n">
-        <v>536.1085951921646</v>
+        <v>977.1315325692362</v>
       </c>
       <c r="H25" t="n">
-        <v>670.1357439902057</v>
+        <v>3132.150960432975</v>
       </c>
       <c r="I25" t="n">
-        <v>1072.217190384329</v>
+        <v>4362.194341826947</v>
       </c>
       <c r="J25" t="n">
         <v>0</v>
@@ -3799,16 +3799,16 @@
         <v>0</v>
       </c>
       <c r="L25" t="n">
-        <v>3184.724508412015</v>
+        <v>2606.863019054845</v>
       </c>
       <c r="M25" t="n">
-        <v>4256.941698796345</v>
+        <v>6969.057360881792</v>
       </c>
       <c r="N25" t="n">
-        <v>74.81249999999999</v>
+        <v>37.40625</v>
       </c>
       <c r="O25" t="n">
-        <v>0.625</v>
+        <v>0.7180218750000001</v>
       </c>
       <c r="P25" t="inlineStr">
         <is>
@@ -3819,7 +3819,7 @@
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>winter</t>
+          <t>summer</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
@@ -3833,40 +3833,40 @@
         </is>
       </c>
       <c r="D26" t="n">
-        <v>-107.5021054623863</v>
+        <v>1594.80446851474</v>
       </c>
       <c r="E26" t="n">
-        <v>162.7794540493492</v>
+        <v>80.93104235922647</v>
       </c>
       <c r="F26" t="n">
-        <v>430.0084218495453</v>
+        <v>2503.231778832977</v>
       </c>
       <c r="G26" t="n">
-        <v>537.5105273119316</v>
+        <v>908.4273103182369</v>
       </c>
       <c r="H26" t="n">
-        <v>634.8524485419251</v>
+        <v>2908.52321900036</v>
       </c>
       <c r="I26" t="n">
-        <v>1075.021054623863</v>
+        <v>4055.479063920699</v>
       </c>
       <c r="J26" t="n">
-        <v>2048.440266923798</v>
+        <v>1501.079408027346</v>
       </c>
       <c r="K26" t="n">
         <v>0</v>
       </c>
       <c r="L26" t="n">
-        <v>1133.480377248684</v>
+        <v>1412.498888933747</v>
       </c>
       <c r="M26" t="n">
-        <v>4256.941698796345</v>
+        <v>6969.057360881792</v>
       </c>
       <c r="N26" t="n">
-        <v>26.62663614982504</v>
+        <v>20.2681484136188</v>
       </c>
       <c r="O26" t="n">
-        <v>0.4000000000000001</v>
+        <v>0.617246875</v>
       </c>
       <c r="P26" t="inlineStr">
         <is>
@@ -3877,7 +3877,7 @@
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>winter</t>
+          <t>summer</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
@@ -3891,40 +3891,40 @@
         </is>
       </c>
       <c r="D27" t="n">
-        <v>-151.43884576145</v>
+        <v>1801.558144695776</v>
       </c>
       <c r="E27" t="n">
-        <v>247.9373608460197</v>
+        <v>100.220475257742</v>
       </c>
       <c r="F27" t="n">
-        <v>605.7553830458008</v>
+        <v>2827.755808470863</v>
       </c>
       <c r="G27" t="n">
-        <v>757.1942288072509</v>
+        <v>1026.197663775088</v>
       </c>
       <c r="H27" t="n">
-        <v>739.7248794041344</v>
+        <v>3050.505808470863</v>
       </c>
       <c r="I27" t="n">
-        <v>1514.388457614502</v>
+        <v>4581.239570424498</v>
       </c>
       <c r="J27" t="n">
-        <v>1339.694963583336</v>
+        <v>825</v>
       </c>
       <c r="K27" t="n">
         <v>0</v>
       </c>
       <c r="L27" t="n">
-        <v>1402.858277598507</v>
+        <v>1562.817790457294</v>
       </c>
       <c r="M27" t="n">
-        <v>4256.941698796345</v>
+        <v>6969.057360881792</v>
       </c>
       <c r="N27" t="n">
-        <v>32.9546039588742</v>
+        <v>22.42509581323853</v>
       </c>
       <c r="O27" t="n">
-        <v>0.4000000000000001</v>
+        <v>0.617246875</v>
       </c>
       <c r="P27" t="inlineStr">
         <is>
@@ -3935,7 +3935,7 @@
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>winter</t>
+          <t>summer</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
@@ -3949,40 +3949,40 @@
         </is>
       </c>
       <c r="D28" t="n">
-        <v>-112.0982459944941</v>
+        <v>1589.759955512711</v>
       </c>
       <c r="E28" t="n">
-        <v>170.8460593499907</v>
+        <v>82.61079165024194</v>
       </c>
       <c r="F28" t="n">
-        <v>448.3929839779769</v>
+        <v>2495.313826817721</v>
       </c>
       <c r="G28" t="n">
-        <v>560.4912299724709</v>
+        <v>905.55387130501</v>
       </c>
       <c r="H28" t="n">
-        <v>645.0983200951496</v>
+        <v>2907.223771468592</v>
       </c>
       <c r="I28" t="n">
-        <v>1120.982459944942</v>
+        <v>4042.65121118308</v>
       </c>
       <c r="J28" t="n">
-        <v>1967.053361171726</v>
+        <v>1525.592387595819</v>
       </c>
       <c r="K28" t="n">
         <v>0</v>
       </c>
       <c r="L28" t="n">
-        <v>1168.905877679676</v>
+        <v>1400.813762102893</v>
       </c>
       <c r="M28" t="n">
-        <v>4256.941698796345</v>
+        <v>6969.057360881792</v>
       </c>
       <c r="N28" t="n">
-        <v>27.45881809962738</v>
+        <v>20.10047685883373</v>
       </c>
       <c r="O28" t="n">
-        <v>0.4000000000000001</v>
+        <v>0.617246875</v>
       </c>
       <c r="P28" t="inlineStr">
         <is>
@@ -3993,7 +3993,7 @@
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>winter</t>
+          <t>summer</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
@@ -4007,40 +4007,40 @@
         </is>
       </c>
       <c r="D29" t="n">
-        <v>-71.17852225581669</v>
+        <v>1290.835619291507</v>
       </c>
       <c r="E29" t="n">
-        <v>103.2601879360226</v>
+        <v>60.31475048610878</v>
       </c>
       <c r="F29" t="n">
-        <v>284.7140890232669</v>
+        <v>2026.117186935999</v>
       </c>
       <c r="G29" t="n">
-        <v>355.8926112790836</v>
+        <v>735.2815676444922</v>
       </c>
       <c r="H29" t="n">
-        <v>558.3173993819255</v>
+        <v>2707.354273530857</v>
       </c>
       <c r="I29" t="n">
-        <v>711.7852225581673</v>
+        <v>3282.506998412911</v>
       </c>
       <c r="J29" t="n">
-        <v>2736.033103586585</v>
+        <v>2523.100320721695</v>
       </c>
       <c r="K29" t="n">
         <v>0</v>
       </c>
       <c r="L29" t="n">
-        <v>809.123372651592</v>
+        <v>1163.450041747187</v>
       </c>
       <c r="M29" t="n">
-        <v>4256.941698796345</v>
+        <v>6969.057360881792</v>
       </c>
       <c r="N29" t="n">
-        <v>19.00715184519376</v>
+        <v>16.6945109144571</v>
       </c>
       <c r="O29" t="n">
-        <v>0.4000000000000001</v>
+        <v>0.617246875</v>
       </c>
       <c r="P29" t="inlineStr">
         <is>
@@ -4051,7 +4051,7 @@
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>winter</t>
+          <t>summer</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
@@ -4065,40 +4065,40 @@
         </is>
       </c>
       <c r="D30" t="n">
-        <v>0</v>
+        <v>196.0634441354357</v>
       </c>
       <c r="E30" t="n">
         <v>0</v>
       </c>
       <c r="F30" t="n">
-        <v>0</v>
+        <v>307.7444625448957</v>
       </c>
       <c r="G30" t="n">
-        <v>0</v>
+        <v>111.68101840946</v>
       </c>
       <c r="H30" t="n">
-        <v>425.6941698796345</v>
+        <v>1982.371748697592</v>
       </c>
       <c r="I30" t="n">
-        <v>0</v>
+        <v>498.575975042232</v>
       </c>
       <c r="J30" t="n">
-        <v>4256.941698796345</v>
+        <v>6202.323282047022</v>
       </c>
       <c r="K30" t="n">
         <v>0</v>
       </c>
       <c r="L30" t="n">
-        <v>0</v>
+        <v>268.1581037925383</v>
       </c>
       <c r="M30" t="n">
-        <v>4256.941698796345</v>
+        <v>6969.057360881792</v>
       </c>
       <c r="N30" t="n">
-        <v>0</v>
+        <v>3.847838953051871</v>
       </c>
       <c r="O30" t="n">
-        <v>0.4000000000000001</v>
+        <v>0.617246875</v>
       </c>
       <c r="P30" t="inlineStr">
         <is>
@@ -4109,7 +4109,7 @@
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>winter</t>
+          <t>summer</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
@@ -4123,22 +4123,22 @@
         </is>
       </c>
       <c r="D31" t="n">
-        <v>-221.8718013412653</v>
+        <v>2043.464328520971</v>
       </c>
       <c r="E31" t="n">
-        <v>365.1888939630039</v>
+        <v>113.6776888270774</v>
       </c>
       <c r="F31" t="n">
-        <v>887.4872053650619</v>
+        <v>3207.455802296059</v>
       </c>
       <c r="G31" t="n">
-        <v>1109.359006706327</v>
+        <v>1163.991473775088</v>
       </c>
       <c r="H31" t="n">
-        <v>887.4872053650619</v>
+        <v>3207.455802296059</v>
       </c>
       <c r="I31" t="n">
-        <v>2218.718013412655</v>
+        <v>5196.390507924498</v>
       </c>
       <c r="J31" t="n">
         <v>0</v>
@@ -4147,16 +4147,16 @@
         <v>0</v>
       </c>
       <c r="L31" t="n">
-        <v>2038.22368538369</v>
+        <v>1772.666852957294</v>
       </c>
       <c r="M31" t="n">
-        <v>4256.941698796345</v>
+        <v>6969.057360881792</v>
       </c>
       <c r="N31" t="n">
-        <v>47.88</v>
+        <v>25.43624999999999</v>
       </c>
       <c r="O31" t="n">
-        <v>0.4000000000000001</v>
+        <v>0.617246875</v>
       </c>
       <c r="P31" t="inlineStr">
         <is>
@@ -4167,7 +4167,7 @@
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>winter</t>
+          <t>summer</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
@@ -4181,40 +4181,40 @@
         </is>
       </c>
       <c r="D32" t="n">
-        <v>52.89703753948382</v>
+        <v>1675.735510873967</v>
       </c>
       <c r="E32" t="n">
-        <v>2.380311047479097</v>
+        <v>0</v>
       </c>
       <c r="F32" t="n">
-        <v>209.6290006194359</v>
+        <v>2416.657070598648</v>
       </c>
       <c r="G32" t="n">
-        <v>156.731963079952</v>
+        <v>740.9215597246817</v>
       </c>
       <c r="H32" t="n">
-        <v>414.4730273118157</v>
+        <v>2821.948510766032</v>
       </c>
       <c r="I32" t="n">
-        <v>313.4639261599041</v>
+        <v>3307.685534485186</v>
       </c>
       <c r="J32" t="n">
-        <v>2048.440266923798</v>
+        <v>1501.079408027346</v>
       </c>
       <c r="K32" t="n">
         <v>0</v>
       </c>
       <c r="L32" t="n">
-        <v>1895.037505712643</v>
+        <v>2160.29241836926</v>
       </c>
       <c r="M32" t="n">
-        <v>4256.941698796345</v>
+        <v>6969.057360881792</v>
       </c>
       <c r="N32" t="n">
-        <v>44.51640731298873</v>
+        <v>30.99834463259346</v>
       </c>
       <c r="O32" t="n">
-        <v>0.6687499999999998</v>
+        <v>0.73061875</v>
       </c>
       <c r="P32" t="inlineStr">
         <is>
@@ -4225,7 +4225,7 @@
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>winter</t>
+          <t>summer</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
@@ -4239,40 +4239,40 @@
         </is>
       </c>
       <c r="D33" t="n">
-        <v>96.49851508456965</v>
+        <v>1901.778619953518</v>
       </c>
       <c r="E33" t="n">
         <v>0</v>
       </c>
       <c r="F33" t="n">
-        <v>382.4200412610722</v>
+        <v>2742.644479872023</v>
       </c>
       <c r="G33" t="n">
-        <v>285.9215261765026</v>
+        <v>840.8658599185048</v>
       </c>
       <c r="H33" t="n">
-        <v>516.3895376194058</v>
+        <v>2965.394479872023</v>
       </c>
       <c r="I33" t="n">
-        <v>571.8430523530053</v>
+        <v>3753.865446064754</v>
       </c>
       <c r="J33" t="n">
-        <v>1339.694963583336</v>
+        <v>825</v>
       </c>
       <c r="K33" t="n">
         <v>0</v>
       </c>
       <c r="L33" t="n">
-        <v>2345.403682860004</v>
+        <v>2390.191914817039</v>
       </c>
       <c r="M33" t="n">
-        <v>4256.941698796345</v>
+        <v>6969.057360881792</v>
       </c>
       <c r="N33" t="n">
-        <v>55.09597849374281</v>
+        <v>34.29720536142364</v>
       </c>
       <c r="O33" t="n">
-        <v>0.6687499999999998</v>
+        <v>0.73061875</v>
       </c>
       <c r="P33" t="inlineStr">
         <is>
@@ -4283,7 +4283,7 @@
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>winter</t>
+          <t>summer</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
@@ -4297,40 +4297,40 @@
         </is>
       </c>
       <c r="D34" t="n">
-        <v>56.63652019519108</v>
+        <v>1672.370747162953</v>
       </c>
       <c r="E34" t="n">
-        <v>2.111293160305593</v>
+        <v>0</v>
       </c>
       <c r="F34" t="n">
-        <v>224.4484318846461</v>
+        <v>2411.804586444467</v>
       </c>
       <c r="G34" t="n">
-        <v>167.811911689455</v>
+        <v>739.4338392815139</v>
       </c>
       <c r="H34" t="n">
-        <v>421.1537680018187</v>
+        <v>2823.714531095338</v>
       </c>
       <c r="I34" t="n">
-        <v>335.62382337891</v>
+        <v>3301.043925363901</v>
       </c>
       <c r="J34" t="n">
-        <v>1967.053361171726</v>
+        <v>1525.592387595819</v>
       </c>
       <c r="K34" t="n">
         <v>0</v>
       </c>
       <c r="L34" t="n">
-        <v>1954.264514245709</v>
+        <v>2142.421047922072</v>
       </c>
       <c r="M34" t="n">
-        <v>4256.941698796345</v>
+        <v>6969.057360881792</v>
       </c>
       <c r="N34" t="n">
-        <v>45.90771151031453</v>
+        <v>30.74190578409864</v>
       </c>
       <c r="O34" t="n">
-        <v>0.6687499999999998</v>
+        <v>0.73061875</v>
       </c>
       <c r="P34" t="inlineStr">
         <is>
@@ -4341,7 +4341,7 @@
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>winter</t>
+          <t>summer</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
@@ -4355,40 +4355,40 @@
         </is>
       </c>
       <c r="D35" t="n">
-        <v>28.3762332941421</v>
+        <v>1350.930742252985</v>
       </c>
       <c r="E35" t="n">
-        <v>3.705432386063777</v>
+        <v>0.2196275246308232</v>
       </c>
       <c r="F35" t="n">
-        <v>112.4539615730816</v>
+        <v>1948.240822593811</v>
       </c>
       <c r="G35" t="n">
-        <v>84.07772827893949</v>
+        <v>597.3100803408257</v>
       </c>
       <c r="H35" t="n">
-        <v>386.0572719317401</v>
+        <v>2629.477909188668</v>
       </c>
       <c r="I35" t="n">
-        <v>168.155456557879</v>
+        <v>2666.5628586644</v>
       </c>
       <c r="J35" t="n">
-        <v>2736.033103586585</v>
+        <v>2523.100320721695</v>
       </c>
       <c r="K35" t="n">
         <v>0</v>
       </c>
       <c r="L35" t="n">
-        <v>1352.75313865188</v>
+        <v>1779.394181495698</v>
       </c>
       <c r="M35" t="n">
-        <v>4256.941698796345</v>
+        <v>6969.057360881792</v>
       </c>
       <c r="N35" t="n">
-        <v>31.77758199118331</v>
+        <v>25.53278139858145</v>
       </c>
       <c r="O35" t="n">
-        <v>0.6687499999999998</v>
+        <v>0.73061875</v>
       </c>
       <c r="P35" t="inlineStr">
         <is>
@@ -4399,7 +4399,7 @@
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>winter</t>
+          <t>summer</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
@@ -4413,40 +4413,40 @@
         </is>
       </c>
       <c r="D36" t="n">
-        <v>0</v>
+        <v>180.6652719552377</v>
       </c>
       <c r="E36" t="n">
-        <v>0</v>
+        <v>15.39817218019797</v>
       </c>
       <c r="F36" t="n">
-        <v>0</v>
+        <v>260.5458940561238</v>
       </c>
       <c r="G36" t="n">
-        <v>0</v>
+        <v>79.88062210088603</v>
       </c>
       <c r="H36" t="n">
-        <v>425.6941698796345</v>
+        <v>1935.17318020882</v>
       </c>
       <c r="I36" t="n">
-        <v>0</v>
+        <v>356.6099200932412</v>
       </c>
       <c r="J36" t="n">
-        <v>4256.941698796345</v>
+        <v>6202.323282047022</v>
       </c>
       <c r="K36" t="n">
         <v>0</v>
       </c>
       <c r="L36" t="n">
-        <v>0</v>
+        <v>410.1241587415291</v>
       </c>
       <c r="M36" t="n">
-        <v>4256.941698796345</v>
+        <v>6969.057360881792</v>
       </c>
       <c r="N36" t="n">
-        <v>0</v>
+        <v>5.884930163491096</v>
       </c>
       <c r="O36" t="n">
-        <v>0.6687499999999998</v>
+        <v>0.73061875</v>
       </c>
       <c r="P36" t="inlineStr">
         <is>
@@ -4457,7 +4457,7 @@
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>winter</t>
+          <t>summer</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
@@ -4471,22 +4471,22 @@
         </is>
       </c>
       <c r="D37" t="n">
-        <v>143.3170926217387</v>
+        <v>2157.142017348049</v>
       </c>
       <c r="E37" t="n">
         <v>0</v>
       </c>
       <c r="F37" t="n">
-        <v>567.9603300194827</v>
+        <v>3110.916057266554</v>
       </c>
       <c r="G37" t="n">
-        <v>424.6432373977441</v>
+        <v>953.7740399185049</v>
       </c>
       <c r="H37" t="n">
-        <v>567.9603300194827</v>
+        <v>3110.916057266554</v>
       </c>
       <c r="I37" t="n">
-        <v>849.2864747954883</v>
+        <v>4257.919821064754</v>
       </c>
       <c r="J37" t="n">
         <v>0</v>
@@ -4495,16 +4495,16 @@
         <v>0</v>
       </c>
       <c r="L37" t="n">
-        <v>3407.655224000856</v>
+        <v>2711.137539817038</v>
       </c>
       <c r="M37" t="n">
-        <v>4256.941698796345</v>
+        <v>6969.057360881792</v>
       </c>
       <c r="N37" t="n">
-        <v>80.049375</v>
+        <v>38.90249999999999</v>
       </c>
       <c r="O37" t="n">
-        <v>0.6687499999999998</v>
+        <v>0.73061875</v>
       </c>
       <c r="P37" t="inlineStr">
         <is>
@@ -4515,7 +4515,7 @@
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>winter</t>
+          <t>summer</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
@@ -4529,40 +4529,40 @@
         </is>
       </c>
       <c r="D38" t="n">
-        <v>54.98937282651542</v>
+        <v>1675.735510873967</v>
       </c>
       <c r="E38" t="n">
-        <v>0.2879757604474946</v>
+        <v>0</v>
       </c>
       <c r="F38" t="n">
-        <v>238.2872822482334</v>
+        <v>2416.657070598648</v>
       </c>
       <c r="G38" t="n">
-        <v>183.2979094217179</v>
+        <v>740.9215597246817</v>
       </c>
       <c r="H38" t="n">
-        <v>443.1313089406132</v>
+        <v>2821.948510766032</v>
       </c>
       <c r="I38" t="n">
-        <v>366.5958188434359</v>
+        <v>3307.685534485186</v>
       </c>
       <c r="J38" t="n">
-        <v>2048.440266923798</v>
+        <v>1501.079408027346</v>
       </c>
       <c r="K38" t="n">
         <v>0</v>
       </c>
       <c r="L38" t="n">
-        <v>1841.905613029111</v>
+        <v>2160.29241836926</v>
       </c>
       <c r="M38" t="n">
-        <v>4256.941698796345</v>
+        <v>6969.057360881792</v>
       </c>
       <c r="N38" t="n">
-        <v>43.26828374346569</v>
+        <v>30.99834463259346</v>
       </c>
       <c r="O38" t="n">
-        <v>0.65</v>
+        <v>0.73061875</v>
       </c>
       <c r="P38" t="inlineStr">
         <is>
@@ -4573,7 +4573,7 @@
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>winter</t>
+          <t>summer</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
@@ -4587,40 +4587,40 @@
         </is>
       </c>
       <c r="D39" t="n">
-        <v>95.64030511731534</v>
+        <v>1901.778619953518</v>
       </c>
       <c r="E39" t="n">
-        <v>0.8582099672543109</v>
+        <v>0</v>
       </c>
       <c r="F39" t="n">
-        <v>414.4413221750328</v>
+        <v>2742.644479872023</v>
       </c>
       <c r="G39" t="n">
-        <v>318.8010170577174</v>
+        <v>840.8658599185048</v>
       </c>
       <c r="H39" t="n">
-        <v>548.4108185333664</v>
+        <v>2965.394479872023</v>
       </c>
       <c r="I39" t="n">
-        <v>637.602034115435</v>
+        <v>3753.865446064754</v>
       </c>
       <c r="J39" t="n">
-        <v>1339.694963583336</v>
+        <v>825</v>
       </c>
       <c r="K39" t="n">
         <v>0</v>
       </c>
       <c r="L39" t="n">
-        <v>2279.644701097574</v>
+        <v>2390.191914817039</v>
       </c>
       <c r="M39" t="n">
-        <v>4256.941698796345</v>
+        <v>6969.057360881792</v>
       </c>
       <c r="N39" t="n">
-        <v>53.55123143317059</v>
+        <v>34.29720536142364</v>
       </c>
       <c r="O39" t="n">
-        <v>0.65</v>
+        <v>0.73061875</v>
       </c>
       <c r="P39" t="inlineStr">
         <is>
@@ -4631,7 +4631,7 @@
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>winter</t>
+          <t>summer</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
@@ -4645,40 +4645,40 @@
         </is>
       </c>
       <c r="D40" t="n">
-        <v>58.56244295927172</v>
+        <v>1672.370747162953</v>
       </c>
       <c r="E40" t="n">
-        <v>0.185370396224954</v>
+        <v>0</v>
       </c>
       <c r="F40" t="n">
-        <v>253.770586156844</v>
+        <v>2411.804586444467</v>
       </c>
       <c r="G40" t="n">
-        <v>195.2081431975723</v>
+        <v>739.4338392815139</v>
       </c>
       <c r="H40" t="n">
-        <v>450.4759222740166</v>
+        <v>2823.714531095338</v>
       </c>
       <c r="I40" t="n">
-        <v>390.4162863951446</v>
+        <v>3301.043925363901</v>
       </c>
       <c r="J40" t="n">
-        <v>1967.053361171726</v>
+        <v>1525.592387595819</v>
       </c>
       <c r="K40" t="n">
         <v>0</v>
       </c>
       <c r="L40" t="n">
-        <v>1899.472051229474</v>
+        <v>2142.421047922072</v>
       </c>
       <c r="M40" t="n">
-        <v>4256.941698796345</v>
+        <v>6969.057360881792</v>
       </c>
       <c r="N40" t="n">
-        <v>44.6205794118945</v>
+        <v>30.74190578409864</v>
       </c>
       <c r="O40" t="n">
-        <v>0.65</v>
+        <v>0.73061875</v>
       </c>
       <c r="P40" t="inlineStr">
         <is>
@@ -4689,7 +4689,7 @@
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>winter</t>
+          <t>summer</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
@@ -4703,40 +4703,40 @@
         </is>
       </c>
       <c r="D41" t="n">
-        <v>30.91246719763835</v>
+        <v>1350.930742252985</v>
       </c>
       <c r="E41" t="n">
-        <v>1.169198482567523</v>
+        <v>0.2196275246308232</v>
       </c>
       <c r="F41" t="n">
-        <v>133.9540245230995</v>
+        <v>1948.240822593811</v>
       </c>
       <c r="G41" t="n">
-        <v>103.0415573254611</v>
+        <v>597.3100803408257</v>
       </c>
       <c r="H41" t="n">
-        <v>407.557334881758</v>
+        <v>2629.477909188668</v>
       </c>
       <c r="I41" t="n">
-        <v>206.0831146509223</v>
+        <v>2666.5628586644</v>
       </c>
       <c r="J41" t="n">
-        <v>2736.033103586585</v>
+        <v>2523.100320721695</v>
       </c>
       <c r="K41" t="n">
         <v>0</v>
       </c>
       <c r="L41" t="n">
-        <v>1314.825480558837</v>
+        <v>1779.394181495698</v>
       </c>
       <c r="M41" t="n">
-        <v>4256.941698796345</v>
+        <v>6969.057360881792</v>
       </c>
       <c r="N41" t="n">
-        <v>30.88662174843986</v>
+        <v>25.53278139858145</v>
       </c>
       <c r="O41" t="n">
-        <v>0.65</v>
+        <v>0.73061875</v>
       </c>
       <c r="P41" t="inlineStr">
         <is>
@@ -4747,7 +4747,7 @@
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>winter</t>
+          <t>summer</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
@@ -4761,40 +4761,40 @@
         </is>
       </c>
       <c r="D42" t="n">
-        <v>0</v>
+        <v>180.6652719552377</v>
       </c>
       <c r="E42" t="n">
-        <v>0</v>
+        <v>15.39817218019797</v>
       </c>
       <c r="F42" t="n">
-        <v>0</v>
+        <v>260.5458940561238</v>
       </c>
       <c r="G42" t="n">
-        <v>0</v>
+        <v>79.88062210088603</v>
       </c>
       <c r="H42" t="n">
-        <v>425.6941698796345</v>
+        <v>1935.17318020882</v>
       </c>
       <c r="I42" t="n">
-        <v>0</v>
+        <v>356.6099200932412</v>
       </c>
       <c r="J42" t="n">
-        <v>4256.941698796345</v>
+        <v>6202.323282047022</v>
       </c>
       <c r="K42" t="n">
         <v>0</v>
       </c>
       <c r="L42" t="n">
-        <v>0</v>
+        <v>410.1241587415291</v>
       </c>
       <c r="M42" t="n">
-        <v>4256.941698796345</v>
+        <v>6969.057360881792</v>
       </c>
       <c r="N42" t="n">
-        <v>0</v>
+        <v>5.884930163491096</v>
       </c>
       <c r="O42" t="n">
-        <v>0.65</v>
+        <v>0.73061875</v>
       </c>
       <c r="P42" t="inlineStr">
         <is>
@@ -4805,7 +4805,7 @@
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>winter</t>
+          <t>summer</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
@@ -4819,22 +4819,22 @@
         </is>
       </c>
       <c r="D43" t="n">
-        <v>141.7242315071773</v>
+        <v>2157.142017348049</v>
       </c>
       <c r="E43" t="n">
-        <v>1.592861114561344</v>
+        <v>0</v>
       </c>
       <c r="F43" t="n">
-        <v>614.1383365311015</v>
+        <v>3110.916057266554</v>
       </c>
       <c r="G43" t="n">
-        <v>472.4141050239242</v>
+        <v>953.7740399185049</v>
       </c>
       <c r="H43" t="n">
-        <v>614.1383365311015</v>
+        <v>3110.916057266554</v>
       </c>
       <c r="I43" t="n">
-        <v>944.8282100478484</v>
+        <v>4257.919821064754</v>
       </c>
       <c r="J43" t="n">
         <v>0</v>
@@ -4843,16 +4843,16 @@
         <v>0</v>
       </c>
       <c r="L43" t="n">
-        <v>3312.113488748496</v>
+        <v>2711.137539817038</v>
       </c>
       <c r="M43" t="n">
-        <v>4256.941698796345</v>
+        <v>6969.057360881792</v>
       </c>
       <c r="N43" t="n">
-        <v>77.80499999999999</v>
+        <v>38.90249999999999</v>
       </c>
       <c r="O43" t="n">
-        <v>0.65</v>
+        <v>0.73061875</v>
       </c>
       <c r="P43" t="inlineStr">
         <is>

</xml_diff>